<commit_message>
Gestores: local de atuação, Etapa 0 reordenada, infraestrutura da rede
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AahsCeqM2DTecRKsTTfJbG
</commit_message>
<xml_diff>
--- a/kobo/gestores_semana2_diagnostico.xlsx
+++ b/kobo/gestores_semana2_diagnostico.xlsx
@@ -608,7 +608,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Nome da escola</t>
+          <t>Nome do local de atuação</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
@@ -636,7 +636,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Código INEP (8 dígitos; deixe em branco se não souber)</t>
+          <t>Código INEP (apenas se for local; 8 dígitos)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
@@ -736,7 +736,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Q2.1. Onde a Educação Ambiental acontece hoje na escola</t>
+          <t>Q2.1. Onde a Educação Ambiental acontece hoje neste local</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
@@ -788,7 +788,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Q2.2. Como caracterizar a institucionalização da Educação Ambiental na escola?</t>
+          <t>Q2.2. Como caracterizar a institucionalização da Educação Ambiental neste local?</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
@@ -1952,7 +1952,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Q2.24. Quais métodos/estratégias a escola já utilizou em práticas de Educação Ambiental?</t>
+          <t>Q2.24. Quais métodos/estratégias o local já utilizou em práticas de Educação Ambiental?</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -2260,7 +2260,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Q2.33. Quão confiante você se sente, como gestor(a), para liderar e apoiar a Educação Ambiental na escola hoje?</t>
+          <t>Q2.33. Quão confiante você se sente, como gestor(a), para liderar e apoiar a Educação Ambiental neste local hoje?</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -3004,7 +3004,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Q2.42. Essa leitura reflete a realidade da escola?</t>
+          <t>Q2.42. Essa leitura reflete a realidade do local?</t>
         </is>
       </c>
       <c r="D98" t="inlineStr"/>
@@ -3460,7 +3460,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Q3.6. Nível de envolvimento das famílias com a escola</t>
+          <t>Q3.6. Nível de envolvimento das famílias com o local</t>
         </is>
       </c>
       <c r="D116" t="inlineStr"/>
@@ -3536,7 +3536,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Q3.8. Frequência de atividades da escola com o território/comunidade</t>
+          <t>Q3.8. Frequência de atividades do local com o território/comunidade</t>
         </is>
       </c>
       <c r="D119" t="inlineStr"/>
@@ -3588,7 +3588,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Q3.10. A escola tem mecanismos de escuta da comunidade?</t>
+          <t>Q3.10. O local tem mecanismos de escuta da comunidade?</t>
         </is>
       </c>
       <c r="D121" t="inlineStr"/>
@@ -3612,7 +3612,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Q3.10a. Quais instâncias de decisão colegiada existem e funcionam na escola?</t>
+          <t>Q3.10a. Quais instâncias de decisão colegiada existem e funcionam neste local?</t>
         </is>
       </c>
       <c r="D122" t="inlineStr"/>
@@ -3720,7 +3720,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Existência, contato, parceria e articulação permanente são níveis diferentes — não confunda um com o outro. Só marque "Parceria" ou "Articulação permanente" se a escola já colabora de fato com esse ator; se ele apenas existe no território ou já houve um contato pontual, isso ainda NÃO é parceria. Use "Adicionar" para registrar um ator por vez.</t>
+          <t>Existência, contato, parceria e articulação permanente são níveis diferentes — não confunda um com o outro. Só marque "Parceria" ou "Articulação permanente" se o local já colabora de fato com esse ator; se ele apenas existe no território ou já houve um contato pontual, isso ainda NÃO é parceria. Use "Adicionar" para registrar um ator por vez.</t>
         </is>
       </c>
       <c r="D126" t="inlineStr"/>
@@ -3984,7 +3984,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>Q3.11. A escola sabe a quem contatar em uma emergência climática?</t>
+          <t>Q3.11. O local sabe a quem contatar em uma emergência climática?</t>
         </is>
       </c>
       <c r="D137" t="inlineStr"/>
@@ -4128,7 +4128,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>Q3.16. Canais de comunicação da escola com a comunidade</t>
+          <t>Q3.16. Canais de comunicação do local com a comunidade</t>
         </is>
       </c>
       <c r="D142" t="inlineStr"/>
@@ -7699,7 +7699,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>Materiais produzidos pela escola</t>
+          <t>Materiais produzidos pelo local</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove grades de contribuições atuais e potenciais; renumera Etapa 3
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AahsCeqM2DTecRKsTTfJbG
</commit_message>
<xml_diff>
--- a/kobo/gestores_semana2_diagnostico.xlsx
+++ b/kobo/gestores_semana2_diagnostico.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J276"/>
+  <dimension ref="A1:J202"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4854,31 +4854,23 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>begin_group</t>
+          <t>select_multiple cat_ator</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>net_atual</t>
+          <t>q3_14</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>Q3.14. Contribuições atuais — o que cada ator parceiro(a) já oferece ao local?</t>
+          <t>Q3.14. Quais atores são prioritários para fortalecer a relação? (NET_PRIORITY_ACTORS)</t>
         </is>
       </c>
       <c r="D168" t="inlineStr"/>
       <c r="E168" t="inlineStr"/>
-      <c r="F168" t="inlineStr">
-        <is>
-          <t>(${net_rel_01} = 'parceria' or ${net_rel_01} = 'articulacao') or (${net_rel_02} = 'parceria' or ${net_rel_02} = 'articulacao') or (${net_rel_03} = 'parceria' or ${net_rel_03} = 'articulacao') or (${net_rel_04} = 'parceria' or ${net_rel_04} = 'articulacao') or (${net_rel_05} = 'parceria' or ${net_rel_05} = 'articulacao') or (${net_rel_06} = 'parceria' or ${net_rel_06} = 'articulacao') or (${net_rel_07} = 'parceria' or ${net_rel_07} = 'articulacao') or (${net_rel_08} = 'parceria' or ${net_rel_08} = 'articulacao') or (${net_rel_09} = 'parceria' or ${net_rel_09} = 'articulacao') or (${net_rel_10} = 'parceria' or ${net_rel_10} = 'articulacao') or (${net_rel_11} = 'parceria' or ${net_rel_11} = 'articulacao') or (${net_rel_12} = 'parceria' or ${net_rel_12} = 'articulacao') or (${net_rel_13} = 'parceria' or ${net_rel_13} = 'articulacao') or (${net_rel_14} = 'parceria' or ${net_rel_14} = 'articulacao') or (${net_rel_15} = 'parceria' or ${net_rel_15} = 'articulacao') or (${net_rel_16} = 'parceria' or ${net_rel_16} = 'articulacao') or (${net_rel_17} = 'parceria' or ${net_rel_17} = 'articulacao') or (${net_rel_18} = 'parceria' or ${net_rel_18} = 'articulacao') or (${net_rel_19} = 'parceria' or ${net_rel_19} = 'articulacao') or (${net_rel_20} = 'parceria' or ${net_rel_20} = 'articulacao') or (${net_rel_21} = 'parceria' or ${net_rel_21} = 'articulacao') or (${net_rel_22} = 'parceria' or ${net_rel_22} = 'articulacao') or (${net_rel_23} = 'parceria' or ${net_rel_23} = 'articulacao') or (${net_rel_24} = 'parceria' or ${net_rel_24} = 'articulacao') or (${net_rel_25} = 'parceria' or ${net_rel_25} = 'articulacao') or (${net_rel_26} = 'parceria' or ${net_rel_26} = 'articulacao') or (${net_rel_27} = 'parceria' or ${net_rel_27} = 'articulacao') or (${net_rel_28} = 'parceria' or ${net_rel_28} = 'articulacao') or (${net_rel_29} = 'parceria' or ${net_rel_29} = 'articulacao') or (${net_rel_30} = 'parceria' or ${net_rel_30} = 'articulacao') or (${net_rel_31} = 'parceria' or ${net_rel_31} = 'articulacao') or (${net_rel_32} = 'parceria' or ${net_rel_32} = 'articulacao') or (${net_rel_33} = 'parceria' or ${net_rel_33} = 'articulacao') or (${net_rel_34} = 'parceria' or ${net_rel_34} = 'articulacao')</t>
-        </is>
-      </c>
-      <c r="G168" t="inlineStr">
-        <is>
-          <t>table-list</t>
-        </is>
-      </c>
+      <c r="F168" t="inlineStr"/>
+      <c r="G168" t="inlineStr"/>
       <c r="H168" t="inlineStr"/>
       <c r="I168" t="inlineStr"/>
       <c r="J168" t="inlineStr"/>
@@ -4886,27 +4878,27 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>select_multiple contrib</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>net_atual_01</t>
+          <t>q3_15</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>Secretaria de Educação</t>
+          <t>Q3.15. Cite o nome do ator mais relevante para o local hoje (ex.: UBS Vila Nova)</t>
         </is>
       </c>
       <c r="D169" t="inlineStr"/>
       <c r="E169" t="inlineStr"/>
-      <c r="F169" t="inlineStr">
-        <is>
-          <t>${net_rel_01} = 'parceria' or ${net_rel_01} = 'articulacao'</t>
-        </is>
-      </c>
-      <c r="G169" t="inlineStr"/>
+      <c r="F169" t="inlineStr"/>
+      <c r="G169" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
       <c r="H169" t="inlineStr"/>
       <c r="I169" t="inlineStr"/>
       <c r="J169" t="inlineStr"/>
@@ -4914,26 +4906,26 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>select_multiple contrib</t>
+          <t>select_one sim_nao_ns</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>net_atual_02</t>
+          <t>q3_16</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>Secretaria de Meio Ambiente</t>
+          <t>Q3.16. O local sabe a quem contatar em uma emergência climática?</t>
         </is>
       </c>
       <c r="D170" t="inlineStr"/>
-      <c r="E170" t="inlineStr"/>
-      <c r="F170" t="inlineStr">
-        <is>
-          <t>${net_rel_02} = 'parceria' or ${net_rel_02} = 'articulacao'</t>
-        </is>
-      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr"/>
       <c r="G170" t="inlineStr"/>
       <c r="H170" t="inlineStr"/>
       <c r="I170" t="inlineStr"/>
@@ -4942,27 +4934,31 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>select_multiple contrib</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>net_atual_03</t>
+          <t>q3_17</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>Defesa Civil</t>
+          <t>Q3.17. Quais são esses contatos?</t>
         </is>
       </c>
       <c r="D171" t="inlineStr"/>
       <c r="E171" t="inlineStr"/>
       <c r="F171" t="inlineStr">
         <is>
-          <t>${net_rel_03} = 'parceria' or ${net_rel_03} = 'articulacao'</t>
-        </is>
-      </c>
-      <c r="G171" t="inlineStr"/>
+          <t>${q3_16}='sim'</t>
+        </is>
+      </c>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
       <c r="H171" t="inlineStr"/>
       <c r="I171" t="inlineStr"/>
       <c r="J171" t="inlineStr"/>
@@ -4970,26 +4966,26 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>select_multiple contrib</t>
+          <t>select_one sim_nao_ns</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>net_atual_04</t>
+          <t>q3_18</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>Secretaria de Saúde</t>
+          <t>Q3.18. Existe um procedimento de emergência definido para eventos climáticos?</t>
         </is>
       </c>
       <c r="D172" t="inlineStr"/>
-      <c r="E172" t="inlineStr"/>
-      <c r="F172" t="inlineStr">
-        <is>
-          <t>${net_rel_04} = 'parceria' or ${net_rel_04} = 'articulacao'</t>
-        </is>
-      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F172" t="inlineStr"/>
       <c r="G172" t="inlineStr"/>
       <c r="H172" t="inlineStr"/>
       <c r="I172" t="inlineStr"/>
@@ -4998,24 +4994,24 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>select_multiple contrib</t>
+          <t>select_one sim_nao_ns</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>net_atual_05</t>
+          <t>q3_19</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>Assistência Social</t>
+          <t>Q3.19. Esse procedimento está documentado/formalizado?</t>
         </is>
       </c>
       <c r="D173" t="inlineStr"/>
       <c r="E173" t="inlineStr"/>
       <c r="F173" t="inlineStr">
         <is>
-          <t>${net_rel_05} = 'parceria' or ${net_rel_05} = 'articulacao'</t>
+          <t>${q3_18}='sim'</t>
         </is>
       </c>
       <c r="G173" t="inlineStr"/>
@@ -5026,27 +5022,27 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>select_multiple contrib</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>net_atual_06</t>
+          <t>q3_20</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>Obras</t>
+          <t>Q3.20. Que ações de preparação já foram feitas (simulados, sinalização, etc.)?</t>
         </is>
       </c>
       <c r="D174" t="inlineStr"/>
       <c r="E174" t="inlineStr"/>
-      <c r="F174" t="inlineStr">
-        <is>
-          <t>${net_rel_06} = 'parceria' or ${net_rel_06} = 'articulacao'</t>
-        </is>
-      </c>
-      <c r="G174" t="inlineStr"/>
+      <c r="F174" t="inlineStr"/>
+      <c r="G174" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
       <c r="H174" t="inlineStr"/>
       <c r="I174" t="inlineStr"/>
       <c r="J174" t="inlineStr"/>
@@ -5054,26 +5050,22 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>select_multiple contrib</t>
+          <t>select_multiple canais</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>net_atual_07</t>
+          <t>q3_21</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>Bombeiros</t>
+          <t>Q3.21. Canais de comunicação do local com a comunidade</t>
         </is>
       </c>
       <c r="D175" t="inlineStr"/>
       <c r="E175" t="inlineStr"/>
-      <c r="F175" t="inlineStr">
-        <is>
-          <t>${net_rel_07} = 'parceria' or ${net_rel_07} = 'articulacao'</t>
-        </is>
-      </c>
+      <c r="F175" t="inlineStr"/>
       <c r="G175" t="inlineStr"/>
       <c r="H175" t="inlineStr"/>
       <c r="I175" t="inlineStr"/>
@@ -5082,24 +5074,24 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>select_multiple contrib</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>net_atual_08</t>
+          <t>q3_21_outro</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>UBS</t>
+          <t>Especifique (Outro)</t>
         </is>
       </c>
       <c r="D176" t="inlineStr"/>
       <c r="E176" t="inlineStr"/>
       <c r="F176" t="inlineStr">
         <is>
-          <t>${net_rel_08} = 'parceria' or ${net_rel_08} = 'articulacao'</t>
+          <t>selected(${q3_21}, 'outro')</t>
         </is>
       </c>
       <c r="G176" t="inlineStr"/>
@@ -5110,26 +5102,22 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>select_multiple contrib</t>
+          <t>select_one suficiente</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>net_atual_09</t>
+          <t>q3_22</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>Vigilância</t>
+          <t>Q3.22. Esses canais seriam suficientes numa emergência?</t>
         </is>
       </c>
       <c r="D177" t="inlineStr"/>
       <c r="E177" t="inlineStr"/>
-      <c r="F177" t="inlineStr">
-        <is>
-          <t>${net_rel_09} = 'parceria' or ${net_rel_09} = 'articulacao'</t>
-        </is>
-      </c>
+      <c r="F177" t="inlineStr"/>
       <c r="G177" t="inlineStr"/>
       <c r="H177" t="inlineStr"/>
       <c r="I177" t="inlineStr"/>
@@ -5138,27 +5126,27 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>select_multiple contrib</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>net_atual_10</t>
+          <t>q3_23</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>Outro (poder público)</t>
+          <t>Q3.23. Algum grupo fica de fora desses canais de comunicação?</t>
         </is>
       </c>
       <c r="D178" t="inlineStr"/>
       <c r="E178" t="inlineStr"/>
-      <c r="F178" t="inlineStr">
-        <is>
-          <t>${net_rel_10} = 'parceria' or ${net_rel_10} = 'articulacao'</t>
-        </is>
-      </c>
-      <c r="G178" t="inlineStr"/>
+      <c r="F178" t="inlineStr"/>
+      <c r="G178" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
       <c r="H178" t="inlineStr"/>
       <c r="I178" t="inlineStr"/>
       <c r="J178" t="inlineStr"/>
@@ -5166,27 +5154,31 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>select_multiple contrib</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>net_atual_11</t>
+          <t>q3_24</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>Universidade</t>
-        </is>
-      </c>
-      <c r="D179" t="inlineStr"/>
+          <t>Q3.24. Que capacidades/conhecimentos a comunidade já possui e podem ser mobilizados?</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>Ex.: conhecimento tradicional sobre o clima local, organização comunitária, mutirões, saberes de manejo.</t>
+        </is>
+      </c>
       <c r="E179" t="inlineStr"/>
-      <c r="F179" t="inlineStr">
-        <is>
-          <t>${net_rel_11} = 'parceria' or ${net_rel_11} = 'articulacao'</t>
-        </is>
-      </c>
-      <c r="G179" t="inlineStr"/>
+      <c r="F179" t="inlineStr"/>
+      <c r="G179" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
       <c r="H179" t="inlineStr"/>
       <c r="I179" t="inlineStr"/>
       <c r="J179" t="inlineStr"/>
@@ -5194,27 +5186,27 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>select_multiple contrib</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>net_atual_12</t>
+          <t>q3_25</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>Instituto Federal</t>
+          <t>Q3.25. Quais dessas capacidades parecem mais estratégicas de fortalecer?</t>
         </is>
       </c>
       <c r="D180" t="inlineStr"/>
       <c r="E180" t="inlineStr"/>
-      <c r="F180" t="inlineStr">
-        <is>
-          <t>${net_rel_12} = 'parceria' or ${net_rel_12} = 'articulacao'</t>
-        </is>
-      </c>
-      <c r="G180" t="inlineStr"/>
+      <c r="F180" t="inlineStr"/>
+      <c r="G180" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
       <c r="H180" t="inlineStr"/>
       <c r="I180" t="inlineStr"/>
       <c r="J180" t="inlineStr"/>
@@ -5222,26 +5214,22 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>select_multiple contrib</t>
+          <t>select_multiple barr_artic</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>net_atual_13</t>
+          <t>q3_26</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>Local técnica</t>
+          <t>Q3.26. Barreiras para articular com atores do território</t>
         </is>
       </c>
       <c r="D181" t="inlineStr"/>
       <c r="E181" t="inlineStr"/>
-      <c r="F181" t="inlineStr">
-        <is>
-          <t>${net_rel_13} = 'parceria' or ${net_rel_13} = 'articulacao'</t>
-        </is>
-      </c>
+      <c r="F181" t="inlineStr"/>
       <c r="G181" t="inlineStr"/>
       <c r="H181" t="inlineStr"/>
       <c r="I181" t="inlineStr"/>
@@ -5250,24 +5238,24 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>select_multiple contrib</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>net_atual_14</t>
+          <t>q3_26_outro</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>Centro de pesquisa</t>
+          <t>Especifique (Outro)</t>
         </is>
       </c>
       <c r="D182" t="inlineStr"/>
       <c r="E182" t="inlineStr"/>
       <c r="F182" t="inlineStr">
         <is>
-          <t>${net_rel_14} = 'parceria' or ${net_rel_14} = 'articulacao'</t>
+          <t>selected(${q3_26}, 'outro')</t>
         </is>
       </c>
       <c r="G182" t="inlineStr"/>
@@ -5278,27 +5266,27 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>select_multiple contrib</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>net_atual_15</t>
+          <t>q3_27</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>Museu</t>
+          <t>Q3.27. Descreva um caso concreto de articulação (bem ou malsucedida) com a comunidade/rede</t>
         </is>
       </c>
       <c r="D183" t="inlineStr"/>
       <c r="E183" t="inlineStr"/>
-      <c r="F183" t="inlineStr">
-        <is>
-          <t>${net_rel_15} = 'parceria' or ${net_rel_15} = 'articulacao'</t>
-        </is>
-      </c>
-      <c r="G183" t="inlineStr"/>
+      <c r="F183" t="inlineStr"/>
+      <c r="G183" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
       <c r="H183" t="inlineStr"/>
       <c r="I183" t="inlineStr"/>
       <c r="J183" t="inlineStr"/>
@@ -5306,27 +5294,31 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>select_multiple contrib</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>net_atual_16</t>
+          <t>q3_28</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>Jardim botânico</t>
+          <t>Q3.28. Quem participou desse caso?</t>
         </is>
       </c>
       <c r="D184" t="inlineStr"/>
       <c r="E184" t="inlineStr"/>
       <c r="F184" t="inlineStr">
         <is>
-          <t>${net_rel_16} = 'parceria' or ${net_rel_16} = 'articulacao'</t>
-        </is>
-      </c>
-      <c r="G184" t="inlineStr"/>
+          <t>${q3_27} != ''</t>
+        </is>
+      </c>
+      <c r="G184" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
       <c r="H184" t="inlineStr"/>
       <c r="I184" t="inlineStr"/>
       <c r="J184" t="inlineStr"/>
@@ -5334,27 +5326,31 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>select_multiple contrib</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>net_atual_17</t>
+          <t>q3_29</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>Outro (educação/ciência)</t>
+          <t>Q3.29. O que funcionou bem?</t>
         </is>
       </c>
       <c r="D185" t="inlineStr"/>
       <c r="E185" t="inlineStr"/>
       <c r="F185" t="inlineStr">
         <is>
-          <t>${net_rel_17} = 'parceria' or ${net_rel_17} = 'articulacao'</t>
-        </is>
-      </c>
-      <c r="G185" t="inlineStr"/>
+          <t>${q3_27} != ''</t>
+        </is>
+      </c>
+      <c r="G185" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
       <c r="H185" t="inlineStr"/>
       <c r="I185" t="inlineStr"/>
       <c r="J185" t="inlineStr"/>
@@ -5362,27 +5358,31 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>select_multiple contrib</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>net_atual_18</t>
+          <t>q3_30</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>Associação de moradores</t>
+          <t>Q3.30. Quais foram as dificuldades?</t>
         </is>
       </c>
       <c r="D186" t="inlineStr"/>
       <c r="E186" t="inlineStr"/>
       <c r="F186" t="inlineStr">
         <is>
-          <t>${net_rel_18} = 'parceria' or ${net_rel_18} = 'articulacao'</t>
-        </is>
-      </c>
-      <c r="G186" t="inlineStr"/>
+          <t>${q3_27} != ''</t>
+        </is>
+      </c>
+      <c r="G186" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
       <c r="H186" t="inlineStr"/>
       <c r="I186" t="inlineStr"/>
       <c r="J186" t="inlineStr"/>
@@ -5390,27 +5390,31 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>select_multiple contrib</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>net_atual_19</t>
+          <t>q3_31</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>ONG</t>
+          <t>Q3.31. O que essa experiência ensinou?</t>
         </is>
       </c>
       <c r="D187" t="inlineStr"/>
       <c r="E187" t="inlineStr"/>
       <c r="F187" t="inlineStr">
         <is>
-          <t>${net_rel_19} = 'parceria' or ${net_rel_19} = 'articulacao'</t>
-        </is>
-      </c>
-      <c r="G187" t="inlineStr"/>
+          <t>${q3_27} != ''</t>
+        </is>
+      </c>
+      <c r="G187" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
       <c r="H187" t="inlineStr"/>
       <c r="I187" t="inlineStr"/>
       <c r="J187" t="inlineStr"/>
@@ -5418,27 +5422,27 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>select_multiple contrib</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>net_atual_20</t>
+          <t>q3_32</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>Cooperativa</t>
+          <t>Q3.32. Se houvesse uma relação prioritária para fortalecer agora, qual seria?</t>
         </is>
       </c>
       <c r="D188" t="inlineStr"/>
       <c r="E188" t="inlineStr"/>
-      <c r="F188" t="inlineStr">
-        <is>
-          <t>${net_rel_20} = 'parceria' or ${net_rel_20} = 'articulacao'</t>
-        </is>
-      </c>
-      <c r="G188" t="inlineStr"/>
+      <c r="F188" t="inlineStr"/>
+      <c r="G188" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
       <c r="H188" t="inlineStr"/>
       <c r="I188" t="inlineStr"/>
       <c r="J188" t="inlineStr"/>
@@ -5446,27 +5450,31 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>select_multiple contrib</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>net_atual_21</t>
+          <t>q3_33</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>Catadores</t>
+          <t>Q3.33. Por quê?</t>
         </is>
       </c>
       <c r="D189" t="inlineStr"/>
       <c r="E189" t="inlineStr"/>
       <c r="F189" t="inlineStr">
         <is>
-          <t>${net_rel_21} = 'parceria' or ${net_rel_21} = 'articulacao'</t>
-        </is>
-      </c>
-      <c r="G189" t="inlineStr"/>
+          <t>${q3_32} != ''</t>
+        </is>
+      </c>
+      <c r="G189" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
       <c r="H189" t="inlineStr"/>
       <c r="I189" t="inlineStr"/>
       <c r="J189" t="inlineStr"/>
@@ -5474,26 +5482,22 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>select_multiple contrib</t>
+          <t>begin_repeat</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>net_atual_22</t>
+          <t>evid_e3</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>Movimentos sociais</t>
+          <t>Evidências — Evidências sobre participação e redes</t>
         </is>
       </c>
       <c r="D190" t="inlineStr"/>
       <c r="E190" t="inlineStr"/>
-      <c r="F190" t="inlineStr">
-        <is>
-          <t>${net_rel_22} = 'parceria' or ${net_rel_22} = 'articulacao'</t>
-        </is>
-      </c>
+      <c r="F190" t="inlineStr"/>
       <c r="G190" t="inlineStr"/>
       <c r="H190" t="inlineStr"/>
       <c r="I190" t="inlineStr"/>
@@ -5502,26 +5506,22 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>select_multiple contrib</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>net_atual_23</t>
+          <t>evid_e3_nota</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>Coletivos</t>
+          <t>Evidências sustentam análises futuras (problemas, prioridades, plano de ação). Registrar não é obrigatório para todo campo, mas fortalece a rastreabilidade do diagnóstico.</t>
         </is>
       </c>
       <c r="D191" t="inlineStr"/>
       <c r="E191" t="inlineStr"/>
-      <c r="F191" t="inlineStr">
-        <is>
-          <t>${net_rel_23} = 'parceria' or ${net_rel_23} = 'articulacao'</t>
-        </is>
-      </c>
+      <c r="F191" t="inlineStr"/>
       <c r="G191" t="inlineStr"/>
       <c r="H191" t="inlineStr"/>
       <c r="I191" t="inlineStr"/>
@@ -5530,26 +5530,22 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>select_multiple contrib</t>
+          <t>select_one tipo_evid</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>net_atual_24</t>
+          <t>evid_e3_tipo</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>Grupos culturais</t>
+          <t>Tipo de evidência</t>
         </is>
       </c>
       <c r="D192" t="inlineStr"/>
       <c r="E192" t="inlineStr"/>
-      <c r="F192" t="inlineStr">
-        <is>
-          <t>${net_rel_24} = 'parceria' or ${net_rel_24} = 'articulacao'</t>
-        </is>
-      </c>
+      <c r="F192" t="inlineStr"/>
       <c r="G192" t="inlineStr"/>
       <c r="H192" t="inlineStr"/>
       <c r="I192" t="inlineStr"/>
@@ -5558,24 +5554,24 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>select_multiple contrib</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>net_atual_25</t>
+          <t>evid_e3_tipo_outro</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>Organizações comunitárias/religiosas</t>
+          <t>Especifique (Outro)</t>
         </is>
       </c>
       <c r="D193" t="inlineStr"/>
       <c r="E193" t="inlineStr"/>
       <c r="F193" t="inlineStr">
         <is>
-          <t>${net_rel_25} = 'parceria' or ${net_rel_25} = 'articulacao'</t>
+          <t>${evid_e3_tipo}='outro'</t>
         </is>
       </c>
       <c r="G193" t="inlineStr"/>
@@ -5586,27 +5582,27 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>select_multiple contrib</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>net_atual_26</t>
+          <t>evid_e3_desc</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>Outro (sociedade civil)</t>
+          <t>Descreva a evidência</t>
         </is>
       </c>
       <c r="D194" t="inlineStr"/>
       <c r="E194" t="inlineStr"/>
-      <c r="F194" t="inlineStr">
-        <is>
-          <t>${net_rel_26} = 'parceria' or ${net_rel_26} = 'articulacao'</t>
-        </is>
-      </c>
-      <c r="G194" t="inlineStr"/>
+      <c r="F194" t="inlineStr"/>
+      <c r="G194" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
       <c r="H194" t="inlineStr"/>
       <c r="I194" t="inlineStr"/>
       <c r="J194" t="inlineStr"/>
@@ -5614,26 +5610,22 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>select_multiple contrib</t>
+          <t>file</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>net_atual_27</t>
+          <t>evid_e3_anexo</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>Povos indígenas</t>
+          <t>Anexo (foto/documento) — opcional</t>
         </is>
       </c>
       <c r="D195" t="inlineStr"/>
       <c r="E195" t="inlineStr"/>
-      <c r="F195" t="inlineStr">
-        <is>
-          <t>${net_rel_27} = 'parceria' or ${net_rel_27} = 'articulacao'</t>
-        </is>
-      </c>
+      <c r="F195" t="inlineStr"/>
       <c r="G195" t="inlineStr"/>
       <c r="H195" t="inlineStr"/>
       <c r="I195" t="inlineStr"/>
@@ -5642,26 +5634,14 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>select_multiple contrib</t>
-        </is>
-      </c>
-      <c r="B196" t="inlineStr">
-        <is>
-          <t>net_atual_28</t>
-        </is>
-      </c>
-      <c r="C196" t="inlineStr">
-        <is>
-          <t>Quilombolas</t>
-        </is>
-      </c>
+          <t>end_repeat</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr"/>
+      <c r="C196" t="inlineStr"/>
       <c r="D196" t="inlineStr"/>
       <c r="E196" t="inlineStr"/>
-      <c r="F196" t="inlineStr">
-        <is>
-          <t>${net_rel_28} = 'parceria' or ${net_rel_28} = 'articulacao'</t>
-        </is>
-      </c>
+      <c r="F196" t="inlineStr"/>
       <c r="G196" t="inlineStr"/>
       <c r="H196" t="inlineStr"/>
       <c r="I196" t="inlineStr"/>
@@ -5670,26 +5650,14 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>select_multiple contrib</t>
-        </is>
-      </c>
-      <c r="B197" t="inlineStr">
-        <is>
-          <t>net_atual_29</t>
-        </is>
-      </c>
-      <c r="C197" t="inlineStr">
-        <is>
-          <t>Agricultores familiares</t>
-        </is>
-      </c>
+          <t>end_group</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr"/>
+      <c r="C197" t="inlineStr"/>
       <c r="D197" t="inlineStr"/>
       <c r="E197" t="inlineStr"/>
-      <c r="F197" t="inlineStr">
-        <is>
-          <t>${net_rel_29} = 'parceria' or ${net_rel_29} = 'articulacao'</t>
-        </is>
-      </c>
+      <c r="F197" t="inlineStr"/>
       <c r="G197" t="inlineStr"/>
       <c r="H197" t="inlineStr"/>
       <c r="I197" t="inlineStr"/>
@@ -5698,26 +5666,22 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>select_multiple contrib</t>
+          <t>begin_group</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>net_atual_30</t>
+          <t>confirmacao</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>Pescadores</t>
+          <t>Confirmação final</t>
         </is>
       </c>
       <c r="D198" t="inlineStr"/>
       <c r="E198" t="inlineStr"/>
-      <c r="F198" t="inlineStr">
-        <is>
-          <t>${net_rel_30} = 'parceria' or ${net_rel_30} = 'articulacao'</t>
-        </is>
-      </c>
+      <c r="F198" t="inlineStr"/>
       <c r="G198" t="inlineStr"/>
       <c r="H198" t="inlineStr"/>
       <c r="I198" t="inlineStr"/>
@@ -5726,26 +5690,22 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>select_multiple contrib</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>net_atual_31</t>
+          <t>confirmacao_msg</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>Comunidades tradicionais</t>
+          <t>Semana 2/5 concluída. Obrigado(a) pela sua participação! Suas respostas ajudam a construir um diagnóstico mais completo. Revise o que respondeu, confirme abaixo e clique em Enviar para concluir. ATENÇÃO: depois de clicar em Enviar, aparecerá a mensagem "Submission successful" e o formulário voltará em branco. Isso significa que suas respostas FORAM ENVIADAS. Não preencha nem envie novamente.</t>
         </is>
       </c>
       <c r="D199" t="inlineStr"/>
       <c r="E199" t="inlineStr"/>
-      <c r="F199" t="inlineStr">
-        <is>
-          <t>${net_rel_31} = 'parceria' or ${net_rel_31} = 'articulacao'</t>
-        </is>
-      </c>
+      <c r="F199" t="inlineStr"/>
       <c r="G199" t="inlineStr"/>
       <c r="H199" t="inlineStr"/>
       <c r="I199" t="inlineStr"/>
@@ -5754,26 +5714,26 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>select_multiple contrib</t>
+          <t>select_one confirmo</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>net_atual_32</t>
+          <t>confirmacao_envio</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>Lideranças</t>
+          <t>Revisei minhas respostas e confirmo o envio.</t>
         </is>
       </c>
       <c r="D200" t="inlineStr"/>
-      <c r="E200" t="inlineStr"/>
-      <c r="F200" t="inlineStr">
-        <is>
-          <t>${net_rel_32} = 'parceria' or ${net_rel_32} = 'articulacao'</t>
-        </is>
-      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F200" t="inlineStr"/>
       <c r="G200" t="inlineStr"/>
       <c r="H200" t="inlineStr"/>
       <c r="I200" t="inlineStr"/>
@@ -5782,26 +5742,14 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>select_multiple contrib</t>
-        </is>
-      </c>
-      <c r="B201" t="inlineStr">
-        <is>
-          <t>net_atual_33</t>
-        </is>
-      </c>
-      <c r="C201" t="inlineStr">
-        <is>
-          <t>Detentores de conhecimentos locais</t>
-        </is>
-      </c>
+          <t>end_group</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr"/>
+      <c r="C201" t="inlineStr"/>
       <c r="D201" t="inlineStr"/>
       <c r="E201" t="inlineStr"/>
-      <c r="F201" t="inlineStr">
-        <is>
-          <t>${net_rel_33} = 'parceria' or ${net_rel_33} = 'articulacao'</t>
-        </is>
-      </c>
+      <c r="F201" t="inlineStr"/>
       <c r="G201" t="inlineStr"/>
       <c r="H201" t="inlineStr"/>
       <c r="I201" t="inlineStr"/>
@@ -5810,2030 +5758,18 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>select_multiple contrib</t>
-        </is>
-      </c>
-      <c r="B202" t="inlineStr">
-        <is>
-          <t>net_atual_34</t>
-        </is>
-      </c>
-      <c r="C202" t="inlineStr">
-        <is>
-          <t>Outro (comunidades e conhecimentos)</t>
-        </is>
-      </c>
+          <t>end_group</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr"/>
+      <c r="C202" t="inlineStr"/>
       <c r="D202" t="inlineStr"/>
       <c r="E202" t="inlineStr"/>
-      <c r="F202" t="inlineStr">
-        <is>
-          <t>${net_rel_34} = 'parceria' or ${net_rel_34} = 'articulacao'</t>
-        </is>
-      </c>
+      <c r="F202" t="inlineStr"/>
       <c r="G202" t="inlineStr"/>
       <c r="H202" t="inlineStr"/>
       <c r="I202" t="inlineStr"/>
       <c r="J202" t="inlineStr"/>
-    </row>
-    <row r="203">
-      <c r="A203" t="inlineStr">
-        <is>
-          <t>end_group</t>
-        </is>
-      </c>
-      <c r="B203" t="inlineStr"/>
-      <c r="C203" t="inlineStr"/>
-      <c r="D203" t="inlineStr"/>
-      <c r="E203" t="inlineStr"/>
-      <c r="F203" t="inlineStr"/>
-      <c r="G203" t="inlineStr"/>
-      <c r="H203" t="inlineStr"/>
-      <c r="I203" t="inlineStr"/>
-      <c r="J203" t="inlineStr"/>
-    </row>
-    <row r="204">
-      <c r="A204" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="B204" t="inlineStr">
-        <is>
-          <t>net_atual_outro</t>
-        </is>
-      </c>
-      <c r="C204" t="inlineStr">
-        <is>
-          <t>Especifique (Outro) — contribuições atuais</t>
-        </is>
-      </c>
-      <c r="D204" t="inlineStr"/>
-      <c r="E204" t="inlineStr"/>
-      <c r="F204" t="inlineStr">
-        <is>
-          <t>selected(${net_atual_01}, 'outro') or selected(${net_atual_02}, 'outro') or selected(${net_atual_03}, 'outro') or selected(${net_atual_04}, 'outro') or selected(${net_atual_05}, 'outro') or selected(${net_atual_06}, 'outro') or selected(${net_atual_07}, 'outro') or selected(${net_atual_08}, 'outro') or selected(${net_atual_09}, 'outro') or selected(${net_atual_10}, 'outro') or selected(${net_atual_11}, 'outro') or selected(${net_atual_12}, 'outro') or selected(${net_atual_13}, 'outro') or selected(${net_atual_14}, 'outro') or selected(${net_atual_15}, 'outro') or selected(${net_atual_16}, 'outro') or selected(${net_atual_17}, 'outro') or selected(${net_atual_18}, 'outro') or selected(${net_atual_19}, 'outro') or selected(${net_atual_20}, 'outro') or selected(${net_atual_21}, 'outro') or selected(${net_atual_22}, 'outro') or selected(${net_atual_23}, 'outro') or selected(${net_atual_24}, 'outro') or selected(${net_atual_25}, 'outro') or selected(${net_atual_26}, 'outro') or selected(${net_atual_27}, 'outro') or selected(${net_atual_28}, 'outro') or selected(${net_atual_29}, 'outro') or selected(${net_atual_30}, 'outro') or selected(${net_atual_31}, 'outro') or selected(${net_atual_32}, 'outro') or selected(${net_atual_33}, 'outro') or selected(${net_atual_34}, 'outro')</t>
-        </is>
-      </c>
-      <c r="G204" t="inlineStr">
-        <is>
-          <t>multiline</t>
-        </is>
-      </c>
-      <c r="H204" t="inlineStr"/>
-      <c r="I204" t="inlineStr"/>
-      <c r="J204" t="inlineStr"/>
-    </row>
-    <row r="205">
-      <c r="A205" t="inlineStr">
-        <is>
-          <t>begin_group</t>
-        </is>
-      </c>
-      <c r="B205" t="inlineStr">
-        <is>
-          <t>net_pot</t>
-        </is>
-      </c>
-      <c r="C205" t="inlineStr">
-        <is>
-          <t>Q3.15. Contribuições potenciais — o que cada ator que existe no território poderia oferecer?</t>
-        </is>
-      </c>
-      <c r="D205" t="inlineStr"/>
-      <c r="E205" t="inlineStr"/>
-      <c r="F205" t="inlineStr">
-        <is>
-          <t>(${net_rel_01} != '' and ${net_rel_01} != 'nao_existe' and ${net_rel_01} != 'nao_sei') or (${net_rel_02} != '' and ${net_rel_02} != 'nao_existe' and ${net_rel_02} != 'nao_sei') or (${net_rel_03} != '' and ${net_rel_03} != 'nao_existe' and ${net_rel_03} != 'nao_sei') or (${net_rel_04} != '' and ${net_rel_04} != 'nao_existe' and ${net_rel_04} != 'nao_sei') or (${net_rel_05} != '' and ${net_rel_05} != 'nao_existe' and ${net_rel_05} != 'nao_sei') or (${net_rel_06} != '' and ${net_rel_06} != 'nao_existe' and ${net_rel_06} != 'nao_sei') or (${net_rel_07} != '' and ${net_rel_07} != 'nao_existe' and ${net_rel_07} != 'nao_sei') or (${net_rel_08} != '' and ${net_rel_08} != 'nao_existe' and ${net_rel_08} != 'nao_sei') or (${net_rel_09} != '' and ${net_rel_09} != 'nao_existe' and ${net_rel_09} != 'nao_sei') or (${net_rel_10} != '' and ${net_rel_10} != 'nao_existe' and ${net_rel_10} != 'nao_sei') or (${net_rel_11} != '' and ${net_rel_11} != 'nao_existe' and ${net_rel_11} != 'nao_sei') or (${net_rel_12} != '' and ${net_rel_12} != 'nao_existe' and ${net_rel_12} != 'nao_sei') or (${net_rel_13} != '' and ${net_rel_13} != 'nao_existe' and ${net_rel_13} != 'nao_sei') or (${net_rel_14} != '' and ${net_rel_14} != 'nao_existe' and ${net_rel_14} != 'nao_sei') or (${net_rel_15} != '' and ${net_rel_15} != 'nao_existe' and ${net_rel_15} != 'nao_sei') or (${net_rel_16} != '' and ${net_rel_16} != 'nao_existe' and ${net_rel_16} != 'nao_sei') or (${net_rel_17} != '' and ${net_rel_17} != 'nao_existe' and ${net_rel_17} != 'nao_sei') or (${net_rel_18} != '' and ${net_rel_18} != 'nao_existe' and ${net_rel_18} != 'nao_sei') or (${net_rel_19} != '' and ${net_rel_19} != 'nao_existe' and ${net_rel_19} != 'nao_sei') or (${net_rel_20} != '' and ${net_rel_20} != 'nao_existe' and ${net_rel_20} != 'nao_sei') or (${net_rel_21} != '' and ${net_rel_21} != 'nao_existe' and ${net_rel_21} != 'nao_sei') or (${net_rel_22} != '' and ${net_rel_22} != 'nao_existe' and ${net_rel_22} != 'nao_sei') or (${net_rel_23} != '' and ${net_rel_23} != 'nao_existe' and ${net_rel_23} != 'nao_sei') or (${net_rel_24} != '' and ${net_rel_24} != 'nao_existe' and ${net_rel_24} != 'nao_sei') or (${net_rel_25} != '' and ${net_rel_25} != 'nao_existe' and ${net_rel_25} != 'nao_sei') or (${net_rel_26} != '' and ${net_rel_26} != 'nao_existe' and ${net_rel_26} != 'nao_sei') or (${net_rel_27} != '' and ${net_rel_27} != 'nao_existe' and ${net_rel_27} != 'nao_sei') or (${net_rel_28} != '' and ${net_rel_28} != 'nao_existe' and ${net_rel_28} != 'nao_sei') or (${net_rel_29} != '' and ${net_rel_29} != 'nao_existe' and ${net_rel_29} != 'nao_sei') or (${net_rel_30} != '' and ${net_rel_30} != 'nao_existe' and ${net_rel_30} != 'nao_sei') or (${net_rel_31} != '' and ${net_rel_31} != 'nao_existe' and ${net_rel_31} != 'nao_sei') or (${net_rel_32} != '' and ${net_rel_32} != 'nao_existe' and ${net_rel_32} != 'nao_sei') or (${net_rel_33} != '' and ${net_rel_33} != 'nao_existe' and ${net_rel_33} != 'nao_sei') or (${net_rel_34} != '' and ${net_rel_34} != 'nao_existe' and ${net_rel_34} != 'nao_sei')</t>
-        </is>
-      </c>
-      <c r="G205" t="inlineStr">
-        <is>
-          <t>table-list</t>
-        </is>
-      </c>
-      <c r="H205" t="inlineStr"/>
-      <c r="I205" t="inlineStr"/>
-      <c r="J205" t="inlineStr"/>
-    </row>
-    <row r="206">
-      <c r="A206" t="inlineStr">
-        <is>
-          <t>select_multiple contrib</t>
-        </is>
-      </c>
-      <c r="B206" t="inlineStr">
-        <is>
-          <t>net_pot_01</t>
-        </is>
-      </c>
-      <c r="C206" t="inlineStr">
-        <is>
-          <t>Secretaria de Educação</t>
-        </is>
-      </c>
-      <c r="D206" t="inlineStr"/>
-      <c r="E206" t="inlineStr"/>
-      <c r="F206" t="inlineStr">
-        <is>
-          <t>${net_rel_01} != '' and ${net_rel_01} != 'nao_existe' and ${net_rel_01} != 'nao_sei'</t>
-        </is>
-      </c>
-      <c r="G206" t="inlineStr"/>
-      <c r="H206" t="inlineStr"/>
-      <c r="I206" t="inlineStr"/>
-      <c r="J206" t="inlineStr"/>
-    </row>
-    <row r="207">
-      <c r="A207" t="inlineStr">
-        <is>
-          <t>select_multiple contrib</t>
-        </is>
-      </c>
-      <c r="B207" t="inlineStr">
-        <is>
-          <t>net_pot_02</t>
-        </is>
-      </c>
-      <c r="C207" t="inlineStr">
-        <is>
-          <t>Secretaria de Meio Ambiente</t>
-        </is>
-      </c>
-      <c r="D207" t="inlineStr"/>
-      <c r="E207" t="inlineStr"/>
-      <c r="F207" t="inlineStr">
-        <is>
-          <t>${net_rel_02} != '' and ${net_rel_02} != 'nao_existe' and ${net_rel_02} != 'nao_sei'</t>
-        </is>
-      </c>
-      <c r="G207" t="inlineStr"/>
-      <c r="H207" t="inlineStr"/>
-      <c r="I207" t="inlineStr"/>
-      <c r="J207" t="inlineStr"/>
-    </row>
-    <row r="208">
-      <c r="A208" t="inlineStr">
-        <is>
-          <t>select_multiple contrib</t>
-        </is>
-      </c>
-      <c r="B208" t="inlineStr">
-        <is>
-          <t>net_pot_03</t>
-        </is>
-      </c>
-      <c r="C208" t="inlineStr">
-        <is>
-          <t>Defesa Civil</t>
-        </is>
-      </c>
-      <c r="D208" t="inlineStr"/>
-      <c r="E208" t="inlineStr"/>
-      <c r="F208" t="inlineStr">
-        <is>
-          <t>${net_rel_03} != '' and ${net_rel_03} != 'nao_existe' and ${net_rel_03} != 'nao_sei'</t>
-        </is>
-      </c>
-      <c r="G208" t="inlineStr"/>
-      <c r="H208" t="inlineStr"/>
-      <c r="I208" t="inlineStr"/>
-      <c r="J208" t="inlineStr"/>
-    </row>
-    <row r="209">
-      <c r="A209" t="inlineStr">
-        <is>
-          <t>select_multiple contrib</t>
-        </is>
-      </c>
-      <c r="B209" t="inlineStr">
-        <is>
-          <t>net_pot_04</t>
-        </is>
-      </c>
-      <c r="C209" t="inlineStr">
-        <is>
-          <t>Secretaria de Saúde</t>
-        </is>
-      </c>
-      <c r="D209" t="inlineStr"/>
-      <c r="E209" t="inlineStr"/>
-      <c r="F209" t="inlineStr">
-        <is>
-          <t>${net_rel_04} != '' and ${net_rel_04} != 'nao_existe' and ${net_rel_04} != 'nao_sei'</t>
-        </is>
-      </c>
-      <c r="G209" t="inlineStr"/>
-      <c r="H209" t="inlineStr"/>
-      <c r="I209" t="inlineStr"/>
-      <c r="J209" t="inlineStr"/>
-    </row>
-    <row r="210">
-      <c r="A210" t="inlineStr">
-        <is>
-          <t>select_multiple contrib</t>
-        </is>
-      </c>
-      <c r="B210" t="inlineStr">
-        <is>
-          <t>net_pot_05</t>
-        </is>
-      </c>
-      <c r="C210" t="inlineStr">
-        <is>
-          <t>Assistência Social</t>
-        </is>
-      </c>
-      <c r="D210" t="inlineStr"/>
-      <c r="E210" t="inlineStr"/>
-      <c r="F210" t="inlineStr">
-        <is>
-          <t>${net_rel_05} != '' and ${net_rel_05} != 'nao_existe' and ${net_rel_05} != 'nao_sei'</t>
-        </is>
-      </c>
-      <c r="G210" t="inlineStr"/>
-      <c r="H210" t="inlineStr"/>
-      <c r="I210" t="inlineStr"/>
-      <c r="J210" t="inlineStr"/>
-    </row>
-    <row r="211">
-      <c r="A211" t="inlineStr">
-        <is>
-          <t>select_multiple contrib</t>
-        </is>
-      </c>
-      <c r="B211" t="inlineStr">
-        <is>
-          <t>net_pot_06</t>
-        </is>
-      </c>
-      <c r="C211" t="inlineStr">
-        <is>
-          <t>Obras</t>
-        </is>
-      </c>
-      <c r="D211" t="inlineStr"/>
-      <c r="E211" t="inlineStr"/>
-      <c r="F211" t="inlineStr">
-        <is>
-          <t>${net_rel_06} != '' and ${net_rel_06} != 'nao_existe' and ${net_rel_06} != 'nao_sei'</t>
-        </is>
-      </c>
-      <c r="G211" t="inlineStr"/>
-      <c r="H211" t="inlineStr"/>
-      <c r="I211" t="inlineStr"/>
-      <c r="J211" t="inlineStr"/>
-    </row>
-    <row r="212">
-      <c r="A212" t="inlineStr">
-        <is>
-          <t>select_multiple contrib</t>
-        </is>
-      </c>
-      <c r="B212" t="inlineStr">
-        <is>
-          <t>net_pot_07</t>
-        </is>
-      </c>
-      <c r="C212" t="inlineStr">
-        <is>
-          <t>Bombeiros</t>
-        </is>
-      </c>
-      <c r="D212" t="inlineStr"/>
-      <c r="E212" t="inlineStr"/>
-      <c r="F212" t="inlineStr">
-        <is>
-          <t>${net_rel_07} != '' and ${net_rel_07} != 'nao_existe' and ${net_rel_07} != 'nao_sei'</t>
-        </is>
-      </c>
-      <c r="G212" t="inlineStr"/>
-      <c r="H212" t="inlineStr"/>
-      <c r="I212" t="inlineStr"/>
-      <c r="J212" t="inlineStr"/>
-    </row>
-    <row r="213">
-      <c r="A213" t="inlineStr">
-        <is>
-          <t>select_multiple contrib</t>
-        </is>
-      </c>
-      <c r="B213" t="inlineStr">
-        <is>
-          <t>net_pot_08</t>
-        </is>
-      </c>
-      <c r="C213" t="inlineStr">
-        <is>
-          <t>UBS</t>
-        </is>
-      </c>
-      <c r="D213" t="inlineStr"/>
-      <c r="E213" t="inlineStr"/>
-      <c r="F213" t="inlineStr">
-        <is>
-          <t>${net_rel_08} != '' and ${net_rel_08} != 'nao_existe' and ${net_rel_08} != 'nao_sei'</t>
-        </is>
-      </c>
-      <c r="G213" t="inlineStr"/>
-      <c r="H213" t="inlineStr"/>
-      <c r="I213" t="inlineStr"/>
-      <c r="J213" t="inlineStr"/>
-    </row>
-    <row r="214">
-      <c r="A214" t="inlineStr">
-        <is>
-          <t>select_multiple contrib</t>
-        </is>
-      </c>
-      <c r="B214" t="inlineStr">
-        <is>
-          <t>net_pot_09</t>
-        </is>
-      </c>
-      <c r="C214" t="inlineStr">
-        <is>
-          <t>Vigilância</t>
-        </is>
-      </c>
-      <c r="D214" t="inlineStr"/>
-      <c r="E214" t="inlineStr"/>
-      <c r="F214" t="inlineStr">
-        <is>
-          <t>${net_rel_09} != '' and ${net_rel_09} != 'nao_existe' and ${net_rel_09} != 'nao_sei'</t>
-        </is>
-      </c>
-      <c r="G214" t="inlineStr"/>
-      <c r="H214" t="inlineStr"/>
-      <c r="I214" t="inlineStr"/>
-      <c r="J214" t="inlineStr"/>
-    </row>
-    <row r="215">
-      <c r="A215" t="inlineStr">
-        <is>
-          <t>select_multiple contrib</t>
-        </is>
-      </c>
-      <c r="B215" t="inlineStr">
-        <is>
-          <t>net_pot_10</t>
-        </is>
-      </c>
-      <c r="C215" t="inlineStr">
-        <is>
-          <t>Outro (poder público)</t>
-        </is>
-      </c>
-      <c r="D215" t="inlineStr"/>
-      <c r="E215" t="inlineStr"/>
-      <c r="F215" t="inlineStr">
-        <is>
-          <t>${net_rel_10} != '' and ${net_rel_10} != 'nao_existe' and ${net_rel_10} != 'nao_sei'</t>
-        </is>
-      </c>
-      <c r="G215" t="inlineStr"/>
-      <c r="H215" t="inlineStr"/>
-      <c r="I215" t="inlineStr"/>
-      <c r="J215" t="inlineStr"/>
-    </row>
-    <row r="216">
-      <c r="A216" t="inlineStr">
-        <is>
-          <t>select_multiple contrib</t>
-        </is>
-      </c>
-      <c r="B216" t="inlineStr">
-        <is>
-          <t>net_pot_11</t>
-        </is>
-      </c>
-      <c r="C216" t="inlineStr">
-        <is>
-          <t>Universidade</t>
-        </is>
-      </c>
-      <c r="D216" t="inlineStr"/>
-      <c r="E216" t="inlineStr"/>
-      <c r="F216" t="inlineStr">
-        <is>
-          <t>${net_rel_11} != '' and ${net_rel_11} != 'nao_existe' and ${net_rel_11} != 'nao_sei'</t>
-        </is>
-      </c>
-      <c r="G216" t="inlineStr"/>
-      <c r="H216" t="inlineStr"/>
-      <c r="I216" t="inlineStr"/>
-      <c r="J216" t="inlineStr"/>
-    </row>
-    <row r="217">
-      <c r="A217" t="inlineStr">
-        <is>
-          <t>select_multiple contrib</t>
-        </is>
-      </c>
-      <c r="B217" t="inlineStr">
-        <is>
-          <t>net_pot_12</t>
-        </is>
-      </c>
-      <c r="C217" t="inlineStr">
-        <is>
-          <t>Instituto Federal</t>
-        </is>
-      </c>
-      <c r="D217" t="inlineStr"/>
-      <c r="E217" t="inlineStr"/>
-      <c r="F217" t="inlineStr">
-        <is>
-          <t>${net_rel_12} != '' and ${net_rel_12} != 'nao_existe' and ${net_rel_12} != 'nao_sei'</t>
-        </is>
-      </c>
-      <c r="G217" t="inlineStr"/>
-      <c r="H217" t="inlineStr"/>
-      <c r="I217" t="inlineStr"/>
-      <c r="J217" t="inlineStr"/>
-    </row>
-    <row r="218">
-      <c r="A218" t="inlineStr">
-        <is>
-          <t>select_multiple contrib</t>
-        </is>
-      </c>
-      <c r="B218" t="inlineStr">
-        <is>
-          <t>net_pot_13</t>
-        </is>
-      </c>
-      <c r="C218" t="inlineStr">
-        <is>
-          <t>Local técnica</t>
-        </is>
-      </c>
-      <c r="D218" t="inlineStr"/>
-      <c r="E218" t="inlineStr"/>
-      <c r="F218" t="inlineStr">
-        <is>
-          <t>${net_rel_13} != '' and ${net_rel_13} != 'nao_existe' and ${net_rel_13} != 'nao_sei'</t>
-        </is>
-      </c>
-      <c r="G218" t="inlineStr"/>
-      <c r="H218" t="inlineStr"/>
-      <c r="I218" t="inlineStr"/>
-      <c r="J218" t="inlineStr"/>
-    </row>
-    <row r="219">
-      <c r="A219" t="inlineStr">
-        <is>
-          <t>select_multiple contrib</t>
-        </is>
-      </c>
-      <c r="B219" t="inlineStr">
-        <is>
-          <t>net_pot_14</t>
-        </is>
-      </c>
-      <c r="C219" t="inlineStr">
-        <is>
-          <t>Centro de pesquisa</t>
-        </is>
-      </c>
-      <c r="D219" t="inlineStr"/>
-      <c r="E219" t="inlineStr"/>
-      <c r="F219" t="inlineStr">
-        <is>
-          <t>${net_rel_14} != '' and ${net_rel_14} != 'nao_existe' and ${net_rel_14} != 'nao_sei'</t>
-        </is>
-      </c>
-      <c r="G219" t="inlineStr"/>
-      <c r="H219" t="inlineStr"/>
-      <c r="I219" t="inlineStr"/>
-      <c r="J219" t="inlineStr"/>
-    </row>
-    <row r="220">
-      <c r="A220" t="inlineStr">
-        <is>
-          <t>select_multiple contrib</t>
-        </is>
-      </c>
-      <c r="B220" t="inlineStr">
-        <is>
-          <t>net_pot_15</t>
-        </is>
-      </c>
-      <c r="C220" t="inlineStr">
-        <is>
-          <t>Museu</t>
-        </is>
-      </c>
-      <c r="D220" t="inlineStr"/>
-      <c r="E220" t="inlineStr"/>
-      <c r="F220" t="inlineStr">
-        <is>
-          <t>${net_rel_15} != '' and ${net_rel_15} != 'nao_existe' and ${net_rel_15} != 'nao_sei'</t>
-        </is>
-      </c>
-      <c r="G220" t="inlineStr"/>
-      <c r="H220" t="inlineStr"/>
-      <c r="I220" t="inlineStr"/>
-      <c r="J220" t="inlineStr"/>
-    </row>
-    <row r="221">
-      <c r="A221" t="inlineStr">
-        <is>
-          <t>select_multiple contrib</t>
-        </is>
-      </c>
-      <c r="B221" t="inlineStr">
-        <is>
-          <t>net_pot_16</t>
-        </is>
-      </c>
-      <c r="C221" t="inlineStr">
-        <is>
-          <t>Jardim botânico</t>
-        </is>
-      </c>
-      <c r="D221" t="inlineStr"/>
-      <c r="E221" t="inlineStr"/>
-      <c r="F221" t="inlineStr">
-        <is>
-          <t>${net_rel_16} != '' and ${net_rel_16} != 'nao_existe' and ${net_rel_16} != 'nao_sei'</t>
-        </is>
-      </c>
-      <c r="G221" t="inlineStr"/>
-      <c r="H221" t="inlineStr"/>
-      <c r="I221" t="inlineStr"/>
-      <c r="J221" t="inlineStr"/>
-    </row>
-    <row r="222">
-      <c r="A222" t="inlineStr">
-        <is>
-          <t>select_multiple contrib</t>
-        </is>
-      </c>
-      <c r="B222" t="inlineStr">
-        <is>
-          <t>net_pot_17</t>
-        </is>
-      </c>
-      <c r="C222" t="inlineStr">
-        <is>
-          <t>Outro (educação/ciência)</t>
-        </is>
-      </c>
-      <c r="D222" t="inlineStr"/>
-      <c r="E222" t="inlineStr"/>
-      <c r="F222" t="inlineStr">
-        <is>
-          <t>${net_rel_17} != '' and ${net_rel_17} != 'nao_existe' and ${net_rel_17} != 'nao_sei'</t>
-        </is>
-      </c>
-      <c r="G222" t="inlineStr"/>
-      <c r="H222" t="inlineStr"/>
-      <c r="I222" t="inlineStr"/>
-      <c r="J222" t="inlineStr"/>
-    </row>
-    <row r="223">
-      <c r="A223" t="inlineStr">
-        <is>
-          <t>select_multiple contrib</t>
-        </is>
-      </c>
-      <c r="B223" t="inlineStr">
-        <is>
-          <t>net_pot_18</t>
-        </is>
-      </c>
-      <c r="C223" t="inlineStr">
-        <is>
-          <t>Associação de moradores</t>
-        </is>
-      </c>
-      <c r="D223" t="inlineStr"/>
-      <c r="E223" t="inlineStr"/>
-      <c r="F223" t="inlineStr">
-        <is>
-          <t>${net_rel_18} != '' and ${net_rel_18} != 'nao_existe' and ${net_rel_18} != 'nao_sei'</t>
-        </is>
-      </c>
-      <c r="G223" t="inlineStr"/>
-      <c r="H223" t="inlineStr"/>
-      <c r="I223" t="inlineStr"/>
-      <c r="J223" t="inlineStr"/>
-    </row>
-    <row r="224">
-      <c r="A224" t="inlineStr">
-        <is>
-          <t>select_multiple contrib</t>
-        </is>
-      </c>
-      <c r="B224" t="inlineStr">
-        <is>
-          <t>net_pot_19</t>
-        </is>
-      </c>
-      <c r="C224" t="inlineStr">
-        <is>
-          <t>ONG</t>
-        </is>
-      </c>
-      <c r="D224" t="inlineStr"/>
-      <c r="E224" t="inlineStr"/>
-      <c r="F224" t="inlineStr">
-        <is>
-          <t>${net_rel_19} != '' and ${net_rel_19} != 'nao_existe' and ${net_rel_19} != 'nao_sei'</t>
-        </is>
-      </c>
-      <c r="G224" t="inlineStr"/>
-      <c r="H224" t="inlineStr"/>
-      <c r="I224" t="inlineStr"/>
-      <c r="J224" t="inlineStr"/>
-    </row>
-    <row r="225">
-      <c r="A225" t="inlineStr">
-        <is>
-          <t>select_multiple contrib</t>
-        </is>
-      </c>
-      <c r="B225" t="inlineStr">
-        <is>
-          <t>net_pot_20</t>
-        </is>
-      </c>
-      <c r="C225" t="inlineStr">
-        <is>
-          <t>Cooperativa</t>
-        </is>
-      </c>
-      <c r="D225" t="inlineStr"/>
-      <c r="E225" t="inlineStr"/>
-      <c r="F225" t="inlineStr">
-        <is>
-          <t>${net_rel_20} != '' and ${net_rel_20} != 'nao_existe' and ${net_rel_20} != 'nao_sei'</t>
-        </is>
-      </c>
-      <c r="G225" t="inlineStr"/>
-      <c r="H225" t="inlineStr"/>
-      <c r="I225" t="inlineStr"/>
-      <c r="J225" t="inlineStr"/>
-    </row>
-    <row r="226">
-      <c r="A226" t="inlineStr">
-        <is>
-          <t>select_multiple contrib</t>
-        </is>
-      </c>
-      <c r="B226" t="inlineStr">
-        <is>
-          <t>net_pot_21</t>
-        </is>
-      </c>
-      <c r="C226" t="inlineStr">
-        <is>
-          <t>Catadores</t>
-        </is>
-      </c>
-      <c r="D226" t="inlineStr"/>
-      <c r="E226" t="inlineStr"/>
-      <c r="F226" t="inlineStr">
-        <is>
-          <t>${net_rel_21} != '' and ${net_rel_21} != 'nao_existe' and ${net_rel_21} != 'nao_sei'</t>
-        </is>
-      </c>
-      <c r="G226" t="inlineStr"/>
-      <c r="H226" t="inlineStr"/>
-      <c r="I226" t="inlineStr"/>
-      <c r="J226" t="inlineStr"/>
-    </row>
-    <row r="227">
-      <c r="A227" t="inlineStr">
-        <is>
-          <t>select_multiple contrib</t>
-        </is>
-      </c>
-      <c r="B227" t="inlineStr">
-        <is>
-          <t>net_pot_22</t>
-        </is>
-      </c>
-      <c r="C227" t="inlineStr">
-        <is>
-          <t>Movimentos sociais</t>
-        </is>
-      </c>
-      <c r="D227" t="inlineStr"/>
-      <c r="E227" t="inlineStr"/>
-      <c r="F227" t="inlineStr">
-        <is>
-          <t>${net_rel_22} != '' and ${net_rel_22} != 'nao_existe' and ${net_rel_22} != 'nao_sei'</t>
-        </is>
-      </c>
-      <c r="G227" t="inlineStr"/>
-      <c r="H227" t="inlineStr"/>
-      <c r="I227" t="inlineStr"/>
-      <c r="J227" t="inlineStr"/>
-    </row>
-    <row r="228">
-      <c r="A228" t="inlineStr">
-        <is>
-          <t>select_multiple contrib</t>
-        </is>
-      </c>
-      <c r="B228" t="inlineStr">
-        <is>
-          <t>net_pot_23</t>
-        </is>
-      </c>
-      <c r="C228" t="inlineStr">
-        <is>
-          <t>Coletivos</t>
-        </is>
-      </c>
-      <c r="D228" t="inlineStr"/>
-      <c r="E228" t="inlineStr"/>
-      <c r="F228" t="inlineStr">
-        <is>
-          <t>${net_rel_23} != '' and ${net_rel_23} != 'nao_existe' and ${net_rel_23} != 'nao_sei'</t>
-        </is>
-      </c>
-      <c r="G228" t="inlineStr"/>
-      <c r="H228" t="inlineStr"/>
-      <c r="I228" t="inlineStr"/>
-      <c r="J228" t="inlineStr"/>
-    </row>
-    <row r="229">
-      <c r="A229" t="inlineStr">
-        <is>
-          <t>select_multiple contrib</t>
-        </is>
-      </c>
-      <c r="B229" t="inlineStr">
-        <is>
-          <t>net_pot_24</t>
-        </is>
-      </c>
-      <c r="C229" t="inlineStr">
-        <is>
-          <t>Grupos culturais</t>
-        </is>
-      </c>
-      <c r="D229" t="inlineStr"/>
-      <c r="E229" t="inlineStr"/>
-      <c r="F229" t="inlineStr">
-        <is>
-          <t>${net_rel_24} != '' and ${net_rel_24} != 'nao_existe' and ${net_rel_24} != 'nao_sei'</t>
-        </is>
-      </c>
-      <c r="G229" t="inlineStr"/>
-      <c r="H229" t="inlineStr"/>
-      <c r="I229" t="inlineStr"/>
-      <c r="J229" t="inlineStr"/>
-    </row>
-    <row r="230">
-      <c r="A230" t="inlineStr">
-        <is>
-          <t>select_multiple contrib</t>
-        </is>
-      </c>
-      <c r="B230" t="inlineStr">
-        <is>
-          <t>net_pot_25</t>
-        </is>
-      </c>
-      <c r="C230" t="inlineStr">
-        <is>
-          <t>Organizações comunitárias/religiosas</t>
-        </is>
-      </c>
-      <c r="D230" t="inlineStr"/>
-      <c r="E230" t="inlineStr"/>
-      <c r="F230" t="inlineStr">
-        <is>
-          <t>${net_rel_25} != '' and ${net_rel_25} != 'nao_existe' and ${net_rel_25} != 'nao_sei'</t>
-        </is>
-      </c>
-      <c r="G230" t="inlineStr"/>
-      <c r="H230" t="inlineStr"/>
-      <c r="I230" t="inlineStr"/>
-      <c r="J230" t="inlineStr"/>
-    </row>
-    <row r="231">
-      <c r="A231" t="inlineStr">
-        <is>
-          <t>select_multiple contrib</t>
-        </is>
-      </c>
-      <c r="B231" t="inlineStr">
-        <is>
-          <t>net_pot_26</t>
-        </is>
-      </c>
-      <c r="C231" t="inlineStr">
-        <is>
-          <t>Outro (sociedade civil)</t>
-        </is>
-      </c>
-      <c r="D231" t="inlineStr"/>
-      <c r="E231" t="inlineStr"/>
-      <c r="F231" t="inlineStr">
-        <is>
-          <t>${net_rel_26} != '' and ${net_rel_26} != 'nao_existe' and ${net_rel_26} != 'nao_sei'</t>
-        </is>
-      </c>
-      <c r="G231" t="inlineStr"/>
-      <c r="H231" t="inlineStr"/>
-      <c r="I231" t="inlineStr"/>
-      <c r="J231" t="inlineStr"/>
-    </row>
-    <row r="232">
-      <c r="A232" t="inlineStr">
-        <is>
-          <t>select_multiple contrib</t>
-        </is>
-      </c>
-      <c r="B232" t="inlineStr">
-        <is>
-          <t>net_pot_27</t>
-        </is>
-      </c>
-      <c r="C232" t="inlineStr">
-        <is>
-          <t>Povos indígenas</t>
-        </is>
-      </c>
-      <c r="D232" t="inlineStr"/>
-      <c r="E232" t="inlineStr"/>
-      <c r="F232" t="inlineStr">
-        <is>
-          <t>${net_rel_27} != '' and ${net_rel_27} != 'nao_existe' and ${net_rel_27} != 'nao_sei'</t>
-        </is>
-      </c>
-      <c r="G232" t="inlineStr"/>
-      <c r="H232" t="inlineStr"/>
-      <c r="I232" t="inlineStr"/>
-      <c r="J232" t="inlineStr"/>
-    </row>
-    <row r="233">
-      <c r="A233" t="inlineStr">
-        <is>
-          <t>select_multiple contrib</t>
-        </is>
-      </c>
-      <c r="B233" t="inlineStr">
-        <is>
-          <t>net_pot_28</t>
-        </is>
-      </c>
-      <c r="C233" t="inlineStr">
-        <is>
-          <t>Quilombolas</t>
-        </is>
-      </c>
-      <c r="D233" t="inlineStr"/>
-      <c r="E233" t="inlineStr"/>
-      <c r="F233" t="inlineStr">
-        <is>
-          <t>${net_rel_28} != '' and ${net_rel_28} != 'nao_existe' and ${net_rel_28} != 'nao_sei'</t>
-        </is>
-      </c>
-      <c r="G233" t="inlineStr"/>
-      <c r="H233" t="inlineStr"/>
-      <c r="I233" t="inlineStr"/>
-      <c r="J233" t="inlineStr"/>
-    </row>
-    <row r="234">
-      <c r="A234" t="inlineStr">
-        <is>
-          <t>select_multiple contrib</t>
-        </is>
-      </c>
-      <c r="B234" t="inlineStr">
-        <is>
-          <t>net_pot_29</t>
-        </is>
-      </c>
-      <c r="C234" t="inlineStr">
-        <is>
-          <t>Agricultores familiares</t>
-        </is>
-      </c>
-      <c r="D234" t="inlineStr"/>
-      <c r="E234" t="inlineStr"/>
-      <c r="F234" t="inlineStr">
-        <is>
-          <t>${net_rel_29} != '' and ${net_rel_29} != 'nao_existe' and ${net_rel_29} != 'nao_sei'</t>
-        </is>
-      </c>
-      <c r="G234" t="inlineStr"/>
-      <c r="H234" t="inlineStr"/>
-      <c r="I234" t="inlineStr"/>
-      <c r="J234" t="inlineStr"/>
-    </row>
-    <row r="235">
-      <c r="A235" t="inlineStr">
-        <is>
-          <t>select_multiple contrib</t>
-        </is>
-      </c>
-      <c r="B235" t="inlineStr">
-        <is>
-          <t>net_pot_30</t>
-        </is>
-      </c>
-      <c r="C235" t="inlineStr">
-        <is>
-          <t>Pescadores</t>
-        </is>
-      </c>
-      <c r="D235" t="inlineStr"/>
-      <c r="E235" t="inlineStr"/>
-      <c r="F235" t="inlineStr">
-        <is>
-          <t>${net_rel_30} != '' and ${net_rel_30} != 'nao_existe' and ${net_rel_30} != 'nao_sei'</t>
-        </is>
-      </c>
-      <c r="G235" t="inlineStr"/>
-      <c r="H235" t="inlineStr"/>
-      <c r="I235" t="inlineStr"/>
-      <c r="J235" t="inlineStr"/>
-    </row>
-    <row r="236">
-      <c r="A236" t="inlineStr">
-        <is>
-          <t>select_multiple contrib</t>
-        </is>
-      </c>
-      <c r="B236" t="inlineStr">
-        <is>
-          <t>net_pot_31</t>
-        </is>
-      </c>
-      <c r="C236" t="inlineStr">
-        <is>
-          <t>Comunidades tradicionais</t>
-        </is>
-      </c>
-      <c r="D236" t="inlineStr"/>
-      <c r="E236" t="inlineStr"/>
-      <c r="F236" t="inlineStr">
-        <is>
-          <t>${net_rel_31} != '' and ${net_rel_31} != 'nao_existe' and ${net_rel_31} != 'nao_sei'</t>
-        </is>
-      </c>
-      <c r="G236" t="inlineStr"/>
-      <c r="H236" t="inlineStr"/>
-      <c r="I236" t="inlineStr"/>
-      <c r="J236" t="inlineStr"/>
-    </row>
-    <row r="237">
-      <c r="A237" t="inlineStr">
-        <is>
-          <t>select_multiple contrib</t>
-        </is>
-      </c>
-      <c r="B237" t="inlineStr">
-        <is>
-          <t>net_pot_32</t>
-        </is>
-      </c>
-      <c r="C237" t="inlineStr">
-        <is>
-          <t>Lideranças</t>
-        </is>
-      </c>
-      <c r="D237" t="inlineStr"/>
-      <c r="E237" t="inlineStr"/>
-      <c r="F237" t="inlineStr">
-        <is>
-          <t>${net_rel_32} != '' and ${net_rel_32} != 'nao_existe' and ${net_rel_32} != 'nao_sei'</t>
-        </is>
-      </c>
-      <c r="G237" t="inlineStr"/>
-      <c r="H237" t="inlineStr"/>
-      <c r="I237" t="inlineStr"/>
-      <c r="J237" t="inlineStr"/>
-    </row>
-    <row r="238">
-      <c r="A238" t="inlineStr">
-        <is>
-          <t>select_multiple contrib</t>
-        </is>
-      </c>
-      <c r="B238" t="inlineStr">
-        <is>
-          <t>net_pot_33</t>
-        </is>
-      </c>
-      <c r="C238" t="inlineStr">
-        <is>
-          <t>Detentores de conhecimentos locais</t>
-        </is>
-      </c>
-      <c r="D238" t="inlineStr"/>
-      <c r="E238" t="inlineStr"/>
-      <c r="F238" t="inlineStr">
-        <is>
-          <t>${net_rel_33} != '' and ${net_rel_33} != 'nao_existe' and ${net_rel_33} != 'nao_sei'</t>
-        </is>
-      </c>
-      <c r="G238" t="inlineStr"/>
-      <c r="H238" t="inlineStr"/>
-      <c r="I238" t="inlineStr"/>
-      <c r="J238" t="inlineStr"/>
-    </row>
-    <row r="239">
-      <c r="A239" t="inlineStr">
-        <is>
-          <t>select_multiple contrib</t>
-        </is>
-      </c>
-      <c r="B239" t="inlineStr">
-        <is>
-          <t>net_pot_34</t>
-        </is>
-      </c>
-      <c r="C239" t="inlineStr">
-        <is>
-          <t>Outro (comunidades e conhecimentos)</t>
-        </is>
-      </c>
-      <c r="D239" t="inlineStr"/>
-      <c r="E239" t="inlineStr"/>
-      <c r="F239" t="inlineStr">
-        <is>
-          <t>${net_rel_34} != '' and ${net_rel_34} != 'nao_existe' and ${net_rel_34} != 'nao_sei'</t>
-        </is>
-      </c>
-      <c r="G239" t="inlineStr"/>
-      <c r="H239" t="inlineStr"/>
-      <c r="I239" t="inlineStr"/>
-      <c r="J239" t="inlineStr"/>
-    </row>
-    <row r="240">
-      <c r="A240" t="inlineStr">
-        <is>
-          <t>end_group</t>
-        </is>
-      </c>
-      <c r="B240" t="inlineStr"/>
-      <c r="C240" t="inlineStr"/>
-      <c r="D240" t="inlineStr"/>
-      <c r="E240" t="inlineStr"/>
-      <c r="F240" t="inlineStr"/>
-      <c r="G240" t="inlineStr"/>
-      <c r="H240" t="inlineStr"/>
-      <c r="I240" t="inlineStr"/>
-      <c r="J240" t="inlineStr"/>
-    </row>
-    <row r="241">
-      <c r="A241" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="B241" t="inlineStr">
-        <is>
-          <t>net_pot_outro</t>
-        </is>
-      </c>
-      <c r="C241" t="inlineStr">
-        <is>
-          <t>Especifique (Outro) — contribuições potenciais</t>
-        </is>
-      </c>
-      <c r="D241" t="inlineStr"/>
-      <c r="E241" t="inlineStr"/>
-      <c r="F241" t="inlineStr">
-        <is>
-          <t>selected(${net_pot_01}, 'outro') or selected(${net_pot_02}, 'outro') or selected(${net_pot_03}, 'outro') or selected(${net_pot_04}, 'outro') or selected(${net_pot_05}, 'outro') or selected(${net_pot_06}, 'outro') or selected(${net_pot_07}, 'outro') or selected(${net_pot_08}, 'outro') or selected(${net_pot_09}, 'outro') or selected(${net_pot_10}, 'outro') or selected(${net_pot_11}, 'outro') or selected(${net_pot_12}, 'outro') or selected(${net_pot_13}, 'outro') or selected(${net_pot_14}, 'outro') or selected(${net_pot_15}, 'outro') or selected(${net_pot_16}, 'outro') or selected(${net_pot_17}, 'outro') or selected(${net_pot_18}, 'outro') or selected(${net_pot_19}, 'outro') or selected(${net_pot_20}, 'outro') or selected(${net_pot_21}, 'outro') or selected(${net_pot_22}, 'outro') or selected(${net_pot_23}, 'outro') or selected(${net_pot_24}, 'outro') or selected(${net_pot_25}, 'outro') or selected(${net_pot_26}, 'outro') or selected(${net_pot_27}, 'outro') or selected(${net_pot_28}, 'outro') or selected(${net_pot_29}, 'outro') or selected(${net_pot_30}, 'outro') or selected(${net_pot_31}, 'outro') or selected(${net_pot_32}, 'outro') or selected(${net_pot_33}, 'outro') or selected(${net_pot_34}, 'outro')</t>
-        </is>
-      </c>
-      <c r="G241" t="inlineStr">
-        <is>
-          <t>multiline</t>
-        </is>
-      </c>
-      <c r="H241" t="inlineStr"/>
-      <c r="I241" t="inlineStr"/>
-      <c r="J241" t="inlineStr"/>
-    </row>
-    <row r="242">
-      <c r="A242" t="inlineStr">
-        <is>
-          <t>select_multiple cat_ator</t>
-        </is>
-      </c>
-      <c r="B242" t="inlineStr">
-        <is>
-          <t>q3_16</t>
-        </is>
-      </c>
-      <c r="C242" t="inlineStr">
-        <is>
-          <t>Q3.16. Quais atores são prioritários para fortalecer a relação? (NET_PRIORITY_ACTORS)</t>
-        </is>
-      </c>
-      <c r="D242" t="inlineStr"/>
-      <c r="E242" t="inlineStr"/>
-      <c r="F242" t="inlineStr"/>
-      <c r="G242" t="inlineStr"/>
-      <c r="H242" t="inlineStr"/>
-      <c r="I242" t="inlineStr"/>
-      <c r="J242" t="inlineStr"/>
-    </row>
-    <row r="243">
-      <c r="A243" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="B243" t="inlineStr">
-        <is>
-          <t>q3_17</t>
-        </is>
-      </c>
-      <c r="C243" t="inlineStr">
-        <is>
-          <t>Q3.17. Cite o nome do ator mais relevante para o local hoje (ex.: UBS Vila Nova)</t>
-        </is>
-      </c>
-      <c r="D243" t="inlineStr"/>
-      <c r="E243" t="inlineStr"/>
-      <c r="F243" t="inlineStr"/>
-      <c r="G243" t="inlineStr">
-        <is>
-          <t>multiline</t>
-        </is>
-      </c>
-      <c r="H243" t="inlineStr"/>
-      <c r="I243" t="inlineStr"/>
-      <c r="J243" t="inlineStr"/>
-    </row>
-    <row r="244">
-      <c r="A244" t="inlineStr">
-        <is>
-          <t>select_one sim_nao_ns</t>
-        </is>
-      </c>
-      <c r="B244" t="inlineStr">
-        <is>
-          <t>q3_18</t>
-        </is>
-      </c>
-      <c r="C244" t="inlineStr">
-        <is>
-          <t>Q3.18. O local sabe a quem contatar em uma emergência climática?</t>
-        </is>
-      </c>
-      <c r="D244" t="inlineStr"/>
-      <c r="E244" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="F244" t="inlineStr"/>
-      <c r="G244" t="inlineStr"/>
-      <c r="H244" t="inlineStr"/>
-      <c r="I244" t="inlineStr"/>
-      <c r="J244" t="inlineStr"/>
-    </row>
-    <row r="245">
-      <c r="A245" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="B245" t="inlineStr">
-        <is>
-          <t>q3_19</t>
-        </is>
-      </c>
-      <c r="C245" t="inlineStr">
-        <is>
-          <t>Q3.19. Quais são esses contatos?</t>
-        </is>
-      </c>
-      <c r="D245" t="inlineStr"/>
-      <c r="E245" t="inlineStr"/>
-      <c r="F245" t="inlineStr">
-        <is>
-          <t>${q3_18}='sim'</t>
-        </is>
-      </c>
-      <c r="G245" t="inlineStr">
-        <is>
-          <t>multiline</t>
-        </is>
-      </c>
-      <c r="H245" t="inlineStr"/>
-      <c r="I245" t="inlineStr"/>
-      <c r="J245" t="inlineStr"/>
-    </row>
-    <row r="246">
-      <c r="A246" t="inlineStr">
-        <is>
-          <t>select_one sim_nao_ns</t>
-        </is>
-      </c>
-      <c r="B246" t="inlineStr">
-        <is>
-          <t>q3_20</t>
-        </is>
-      </c>
-      <c r="C246" t="inlineStr">
-        <is>
-          <t>Q3.20. Existe um procedimento de emergência definido para eventos climáticos?</t>
-        </is>
-      </c>
-      <c r="D246" t="inlineStr"/>
-      <c r="E246" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="F246" t="inlineStr"/>
-      <c r="G246" t="inlineStr"/>
-      <c r="H246" t="inlineStr"/>
-      <c r="I246" t="inlineStr"/>
-      <c r="J246" t="inlineStr"/>
-    </row>
-    <row r="247">
-      <c r="A247" t="inlineStr">
-        <is>
-          <t>select_one sim_nao_ns</t>
-        </is>
-      </c>
-      <c r="B247" t="inlineStr">
-        <is>
-          <t>q3_21</t>
-        </is>
-      </c>
-      <c r="C247" t="inlineStr">
-        <is>
-          <t>Q3.21. Esse procedimento está documentado/formalizado?</t>
-        </is>
-      </c>
-      <c r="D247" t="inlineStr"/>
-      <c r="E247" t="inlineStr"/>
-      <c r="F247" t="inlineStr">
-        <is>
-          <t>${q3_20}='sim'</t>
-        </is>
-      </c>
-      <c r="G247" t="inlineStr"/>
-      <c r="H247" t="inlineStr"/>
-      <c r="I247" t="inlineStr"/>
-      <c r="J247" t="inlineStr"/>
-    </row>
-    <row r="248">
-      <c r="A248" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="B248" t="inlineStr">
-        <is>
-          <t>q3_22</t>
-        </is>
-      </c>
-      <c r="C248" t="inlineStr">
-        <is>
-          <t>Q3.22. Que ações de preparação já foram feitas (simulados, sinalização, etc.)?</t>
-        </is>
-      </c>
-      <c r="D248" t="inlineStr"/>
-      <c r="E248" t="inlineStr"/>
-      <c r="F248" t="inlineStr"/>
-      <c r="G248" t="inlineStr">
-        <is>
-          <t>multiline</t>
-        </is>
-      </c>
-      <c r="H248" t="inlineStr"/>
-      <c r="I248" t="inlineStr"/>
-      <c r="J248" t="inlineStr"/>
-    </row>
-    <row r="249">
-      <c r="A249" t="inlineStr">
-        <is>
-          <t>select_multiple canais</t>
-        </is>
-      </c>
-      <c r="B249" t="inlineStr">
-        <is>
-          <t>q3_23</t>
-        </is>
-      </c>
-      <c r="C249" t="inlineStr">
-        <is>
-          <t>Q3.23. Canais de comunicação do local com a comunidade</t>
-        </is>
-      </c>
-      <c r="D249" t="inlineStr"/>
-      <c r="E249" t="inlineStr"/>
-      <c r="F249" t="inlineStr"/>
-      <c r="G249" t="inlineStr"/>
-      <c r="H249" t="inlineStr"/>
-      <c r="I249" t="inlineStr"/>
-      <c r="J249" t="inlineStr"/>
-    </row>
-    <row r="250">
-      <c r="A250" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="B250" t="inlineStr">
-        <is>
-          <t>q3_23_outro</t>
-        </is>
-      </c>
-      <c r="C250" t="inlineStr">
-        <is>
-          <t>Especifique (Outro)</t>
-        </is>
-      </c>
-      <c r="D250" t="inlineStr"/>
-      <c r="E250" t="inlineStr"/>
-      <c r="F250" t="inlineStr">
-        <is>
-          <t>selected(${q3_23}, 'outro')</t>
-        </is>
-      </c>
-      <c r="G250" t="inlineStr"/>
-      <c r="H250" t="inlineStr"/>
-      <c r="I250" t="inlineStr"/>
-      <c r="J250" t="inlineStr"/>
-    </row>
-    <row r="251">
-      <c r="A251" t="inlineStr">
-        <is>
-          <t>select_one suficiente</t>
-        </is>
-      </c>
-      <c r="B251" t="inlineStr">
-        <is>
-          <t>q3_24</t>
-        </is>
-      </c>
-      <c r="C251" t="inlineStr">
-        <is>
-          <t>Q3.24. Esses canais seriam suficientes numa emergência?</t>
-        </is>
-      </c>
-      <c r="D251" t="inlineStr"/>
-      <c r="E251" t="inlineStr"/>
-      <c r="F251" t="inlineStr"/>
-      <c r="G251" t="inlineStr"/>
-      <c r="H251" t="inlineStr"/>
-      <c r="I251" t="inlineStr"/>
-      <c r="J251" t="inlineStr"/>
-    </row>
-    <row r="252">
-      <c r="A252" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="B252" t="inlineStr">
-        <is>
-          <t>q3_25</t>
-        </is>
-      </c>
-      <c r="C252" t="inlineStr">
-        <is>
-          <t>Q3.25. Algum grupo fica de fora desses canais de comunicação?</t>
-        </is>
-      </c>
-      <c r="D252" t="inlineStr"/>
-      <c r="E252" t="inlineStr"/>
-      <c r="F252" t="inlineStr"/>
-      <c r="G252" t="inlineStr">
-        <is>
-          <t>multiline</t>
-        </is>
-      </c>
-      <c r="H252" t="inlineStr"/>
-      <c r="I252" t="inlineStr"/>
-      <c r="J252" t="inlineStr"/>
-    </row>
-    <row r="253">
-      <c r="A253" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="B253" t="inlineStr">
-        <is>
-          <t>q3_26</t>
-        </is>
-      </c>
-      <c r="C253" t="inlineStr">
-        <is>
-          <t>Q3.26. Que capacidades/conhecimentos a comunidade já possui e podem ser mobilizados?</t>
-        </is>
-      </c>
-      <c r="D253" t="inlineStr">
-        <is>
-          <t>Ex.: conhecimento tradicional sobre o clima local, organização comunitária, mutirões, saberes de manejo.</t>
-        </is>
-      </c>
-      <c r="E253" t="inlineStr"/>
-      <c r="F253" t="inlineStr"/>
-      <c r="G253" t="inlineStr">
-        <is>
-          <t>multiline</t>
-        </is>
-      </c>
-      <c r="H253" t="inlineStr"/>
-      <c r="I253" t="inlineStr"/>
-      <c r="J253" t="inlineStr"/>
-    </row>
-    <row r="254">
-      <c r="A254" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="B254" t="inlineStr">
-        <is>
-          <t>q3_27</t>
-        </is>
-      </c>
-      <c r="C254" t="inlineStr">
-        <is>
-          <t>Q3.27. Quais dessas capacidades parecem mais estratégicas de fortalecer?</t>
-        </is>
-      </c>
-      <c r="D254" t="inlineStr"/>
-      <c r="E254" t="inlineStr"/>
-      <c r="F254" t="inlineStr"/>
-      <c r="G254" t="inlineStr">
-        <is>
-          <t>multiline</t>
-        </is>
-      </c>
-      <c r="H254" t="inlineStr"/>
-      <c r="I254" t="inlineStr"/>
-      <c r="J254" t="inlineStr"/>
-    </row>
-    <row r="255">
-      <c r="A255" t="inlineStr">
-        <is>
-          <t>select_multiple barr_artic</t>
-        </is>
-      </c>
-      <c r="B255" t="inlineStr">
-        <is>
-          <t>q3_28</t>
-        </is>
-      </c>
-      <c r="C255" t="inlineStr">
-        <is>
-          <t>Q3.28. Barreiras para articular com atores do território</t>
-        </is>
-      </c>
-      <c r="D255" t="inlineStr"/>
-      <c r="E255" t="inlineStr"/>
-      <c r="F255" t="inlineStr"/>
-      <c r="G255" t="inlineStr"/>
-      <c r="H255" t="inlineStr"/>
-      <c r="I255" t="inlineStr"/>
-      <c r="J255" t="inlineStr"/>
-    </row>
-    <row r="256">
-      <c r="A256" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="B256" t="inlineStr">
-        <is>
-          <t>q3_28_outro</t>
-        </is>
-      </c>
-      <c r="C256" t="inlineStr">
-        <is>
-          <t>Especifique (Outro)</t>
-        </is>
-      </c>
-      <c r="D256" t="inlineStr"/>
-      <c r="E256" t="inlineStr"/>
-      <c r="F256" t="inlineStr">
-        <is>
-          <t>selected(${q3_28}, 'outro')</t>
-        </is>
-      </c>
-      <c r="G256" t="inlineStr"/>
-      <c r="H256" t="inlineStr"/>
-      <c r="I256" t="inlineStr"/>
-      <c r="J256" t="inlineStr"/>
-    </row>
-    <row r="257">
-      <c r="A257" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="B257" t="inlineStr">
-        <is>
-          <t>q3_29</t>
-        </is>
-      </c>
-      <c r="C257" t="inlineStr">
-        <is>
-          <t>Q3.29. Descreva um caso concreto de articulação (bem ou malsucedida) com a comunidade/rede</t>
-        </is>
-      </c>
-      <c r="D257" t="inlineStr"/>
-      <c r="E257" t="inlineStr"/>
-      <c r="F257" t="inlineStr"/>
-      <c r="G257" t="inlineStr">
-        <is>
-          <t>multiline</t>
-        </is>
-      </c>
-      <c r="H257" t="inlineStr"/>
-      <c r="I257" t="inlineStr"/>
-      <c r="J257" t="inlineStr"/>
-    </row>
-    <row r="258">
-      <c r="A258" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="B258" t="inlineStr">
-        <is>
-          <t>q3_30</t>
-        </is>
-      </c>
-      <c r="C258" t="inlineStr">
-        <is>
-          <t>Q3.30. Quem participou desse caso?</t>
-        </is>
-      </c>
-      <c r="D258" t="inlineStr"/>
-      <c r="E258" t="inlineStr"/>
-      <c r="F258" t="inlineStr">
-        <is>
-          <t>${q3_29} != ''</t>
-        </is>
-      </c>
-      <c r="G258" t="inlineStr">
-        <is>
-          <t>multiline</t>
-        </is>
-      </c>
-      <c r="H258" t="inlineStr"/>
-      <c r="I258" t="inlineStr"/>
-      <c r="J258" t="inlineStr"/>
-    </row>
-    <row r="259">
-      <c r="A259" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="B259" t="inlineStr">
-        <is>
-          <t>q3_31</t>
-        </is>
-      </c>
-      <c r="C259" t="inlineStr">
-        <is>
-          <t>Q3.31. O que funcionou bem?</t>
-        </is>
-      </c>
-      <c r="D259" t="inlineStr"/>
-      <c r="E259" t="inlineStr"/>
-      <c r="F259" t="inlineStr">
-        <is>
-          <t>${q3_29} != ''</t>
-        </is>
-      </c>
-      <c r="G259" t="inlineStr">
-        <is>
-          <t>multiline</t>
-        </is>
-      </c>
-      <c r="H259" t="inlineStr"/>
-      <c r="I259" t="inlineStr"/>
-      <c r="J259" t="inlineStr"/>
-    </row>
-    <row r="260">
-      <c r="A260" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="B260" t="inlineStr">
-        <is>
-          <t>q3_32</t>
-        </is>
-      </c>
-      <c r="C260" t="inlineStr">
-        <is>
-          <t>Q3.32. Quais foram as dificuldades?</t>
-        </is>
-      </c>
-      <c r="D260" t="inlineStr"/>
-      <c r="E260" t="inlineStr"/>
-      <c r="F260" t="inlineStr">
-        <is>
-          <t>${q3_29} != ''</t>
-        </is>
-      </c>
-      <c r="G260" t="inlineStr">
-        <is>
-          <t>multiline</t>
-        </is>
-      </c>
-      <c r="H260" t="inlineStr"/>
-      <c r="I260" t="inlineStr"/>
-      <c r="J260" t="inlineStr"/>
-    </row>
-    <row r="261">
-      <c r="A261" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="B261" t="inlineStr">
-        <is>
-          <t>q3_33</t>
-        </is>
-      </c>
-      <c r="C261" t="inlineStr">
-        <is>
-          <t>Q3.33. O que essa experiência ensinou?</t>
-        </is>
-      </c>
-      <c r="D261" t="inlineStr"/>
-      <c r="E261" t="inlineStr"/>
-      <c r="F261" t="inlineStr">
-        <is>
-          <t>${q3_29} != ''</t>
-        </is>
-      </c>
-      <c r="G261" t="inlineStr">
-        <is>
-          <t>multiline</t>
-        </is>
-      </c>
-      <c r="H261" t="inlineStr"/>
-      <c r="I261" t="inlineStr"/>
-      <c r="J261" t="inlineStr"/>
-    </row>
-    <row r="262">
-      <c r="A262" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="B262" t="inlineStr">
-        <is>
-          <t>q3_34</t>
-        </is>
-      </c>
-      <c r="C262" t="inlineStr">
-        <is>
-          <t>Q3.34. Se houvesse uma relação prioritária para fortalecer agora, qual seria?</t>
-        </is>
-      </c>
-      <c r="D262" t="inlineStr"/>
-      <c r="E262" t="inlineStr"/>
-      <c r="F262" t="inlineStr"/>
-      <c r="G262" t="inlineStr">
-        <is>
-          <t>multiline</t>
-        </is>
-      </c>
-      <c r="H262" t="inlineStr"/>
-      <c r="I262" t="inlineStr"/>
-      <c r="J262" t="inlineStr"/>
-    </row>
-    <row r="263">
-      <c r="A263" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="B263" t="inlineStr">
-        <is>
-          <t>q3_35</t>
-        </is>
-      </c>
-      <c r="C263" t="inlineStr">
-        <is>
-          <t>Q3.35. Por quê?</t>
-        </is>
-      </c>
-      <c r="D263" t="inlineStr"/>
-      <c r="E263" t="inlineStr"/>
-      <c r="F263" t="inlineStr">
-        <is>
-          <t>${q3_34} != ''</t>
-        </is>
-      </c>
-      <c r="G263" t="inlineStr">
-        <is>
-          <t>multiline</t>
-        </is>
-      </c>
-      <c r="H263" t="inlineStr"/>
-      <c r="I263" t="inlineStr"/>
-      <c r="J263" t="inlineStr"/>
-    </row>
-    <row r="264">
-      <c r="A264" t="inlineStr">
-        <is>
-          <t>begin_repeat</t>
-        </is>
-      </c>
-      <c r="B264" t="inlineStr">
-        <is>
-          <t>evid_e3</t>
-        </is>
-      </c>
-      <c r="C264" t="inlineStr">
-        <is>
-          <t>Evidências — Evidências sobre participação e redes</t>
-        </is>
-      </c>
-      <c r="D264" t="inlineStr"/>
-      <c r="E264" t="inlineStr"/>
-      <c r="F264" t="inlineStr"/>
-      <c r="G264" t="inlineStr"/>
-      <c r="H264" t="inlineStr"/>
-      <c r="I264" t="inlineStr"/>
-      <c r="J264" t="inlineStr"/>
-    </row>
-    <row r="265">
-      <c r="A265" t="inlineStr">
-        <is>
-          <t>note</t>
-        </is>
-      </c>
-      <c r="B265" t="inlineStr">
-        <is>
-          <t>evid_e3_nota</t>
-        </is>
-      </c>
-      <c r="C265" t="inlineStr">
-        <is>
-          <t>Evidências sustentam análises futuras (problemas, prioridades, plano de ação). Registrar não é obrigatório para todo campo, mas fortalece a rastreabilidade do diagnóstico.</t>
-        </is>
-      </c>
-      <c r="D265" t="inlineStr"/>
-      <c r="E265" t="inlineStr"/>
-      <c r="F265" t="inlineStr"/>
-      <c r="G265" t="inlineStr"/>
-      <c r="H265" t="inlineStr"/>
-      <c r="I265" t="inlineStr"/>
-      <c r="J265" t="inlineStr"/>
-    </row>
-    <row r="266">
-      <c r="A266" t="inlineStr">
-        <is>
-          <t>select_one tipo_evid</t>
-        </is>
-      </c>
-      <c r="B266" t="inlineStr">
-        <is>
-          <t>evid_e3_tipo</t>
-        </is>
-      </c>
-      <c r="C266" t="inlineStr">
-        <is>
-          <t>Tipo de evidência</t>
-        </is>
-      </c>
-      <c r="D266" t="inlineStr"/>
-      <c r="E266" t="inlineStr"/>
-      <c r="F266" t="inlineStr"/>
-      <c r="G266" t="inlineStr"/>
-      <c r="H266" t="inlineStr"/>
-      <c r="I266" t="inlineStr"/>
-      <c r="J266" t="inlineStr"/>
-    </row>
-    <row r="267">
-      <c r="A267" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="B267" t="inlineStr">
-        <is>
-          <t>evid_e3_tipo_outro</t>
-        </is>
-      </c>
-      <c r="C267" t="inlineStr">
-        <is>
-          <t>Especifique (Outro)</t>
-        </is>
-      </c>
-      <c r="D267" t="inlineStr"/>
-      <c r="E267" t="inlineStr"/>
-      <c r="F267" t="inlineStr">
-        <is>
-          <t>${evid_e3_tipo}='outro'</t>
-        </is>
-      </c>
-      <c r="G267" t="inlineStr"/>
-      <c r="H267" t="inlineStr"/>
-      <c r="I267" t="inlineStr"/>
-      <c r="J267" t="inlineStr"/>
-    </row>
-    <row r="268">
-      <c r="A268" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="B268" t="inlineStr">
-        <is>
-          <t>evid_e3_desc</t>
-        </is>
-      </c>
-      <c r="C268" t="inlineStr">
-        <is>
-          <t>Descreva a evidência</t>
-        </is>
-      </c>
-      <c r="D268" t="inlineStr"/>
-      <c r="E268" t="inlineStr"/>
-      <c r="F268" t="inlineStr"/>
-      <c r="G268" t="inlineStr">
-        <is>
-          <t>multiline</t>
-        </is>
-      </c>
-      <c r="H268" t="inlineStr"/>
-      <c r="I268" t="inlineStr"/>
-      <c r="J268" t="inlineStr"/>
-    </row>
-    <row r="269">
-      <c r="A269" t="inlineStr">
-        <is>
-          <t>file</t>
-        </is>
-      </c>
-      <c r="B269" t="inlineStr">
-        <is>
-          <t>evid_e3_anexo</t>
-        </is>
-      </c>
-      <c r="C269" t="inlineStr">
-        <is>
-          <t>Anexo (foto/documento) — opcional</t>
-        </is>
-      </c>
-      <c r="D269" t="inlineStr"/>
-      <c r="E269" t="inlineStr"/>
-      <c r="F269" t="inlineStr"/>
-      <c r="G269" t="inlineStr"/>
-      <c r="H269" t="inlineStr"/>
-      <c r="I269" t="inlineStr"/>
-      <c r="J269" t="inlineStr"/>
-    </row>
-    <row r="270">
-      <c r="A270" t="inlineStr">
-        <is>
-          <t>end_repeat</t>
-        </is>
-      </c>
-      <c r="B270" t="inlineStr"/>
-      <c r="C270" t="inlineStr"/>
-      <c r="D270" t="inlineStr"/>
-      <c r="E270" t="inlineStr"/>
-      <c r="F270" t="inlineStr"/>
-      <c r="G270" t="inlineStr"/>
-      <c r="H270" t="inlineStr"/>
-      <c r="I270" t="inlineStr"/>
-      <c r="J270" t="inlineStr"/>
-    </row>
-    <row r="271">
-      <c r="A271" t="inlineStr">
-        <is>
-          <t>end_group</t>
-        </is>
-      </c>
-      <c r="B271" t="inlineStr"/>
-      <c r="C271" t="inlineStr"/>
-      <c r="D271" t="inlineStr"/>
-      <c r="E271" t="inlineStr"/>
-      <c r="F271" t="inlineStr"/>
-      <c r="G271" t="inlineStr"/>
-      <c r="H271" t="inlineStr"/>
-      <c r="I271" t="inlineStr"/>
-      <c r="J271" t="inlineStr"/>
-    </row>
-    <row r="272">
-      <c r="A272" t="inlineStr">
-        <is>
-          <t>begin_group</t>
-        </is>
-      </c>
-      <c r="B272" t="inlineStr">
-        <is>
-          <t>confirmacao</t>
-        </is>
-      </c>
-      <c r="C272" t="inlineStr">
-        <is>
-          <t>Confirmação final</t>
-        </is>
-      </c>
-      <c r="D272" t="inlineStr"/>
-      <c r="E272" t="inlineStr"/>
-      <c r="F272" t="inlineStr"/>
-      <c r="G272" t="inlineStr"/>
-      <c r="H272" t="inlineStr"/>
-      <c r="I272" t="inlineStr"/>
-      <c r="J272" t="inlineStr"/>
-    </row>
-    <row r="273">
-      <c r="A273" t="inlineStr">
-        <is>
-          <t>note</t>
-        </is>
-      </c>
-      <c r="B273" t="inlineStr">
-        <is>
-          <t>confirmacao_msg</t>
-        </is>
-      </c>
-      <c r="C273" t="inlineStr">
-        <is>
-          <t>Semana 2/5 concluída. Obrigado(a) pela sua participação! Suas respostas ajudam a construir um diagnóstico mais completo. Revise o que respondeu, confirme abaixo e clique em Enviar para concluir. ATENÇÃO: depois de clicar em Enviar, aparecerá a mensagem "Submission successful" e o formulário voltará em branco. Isso significa que suas respostas FORAM ENVIADAS. Não preencha nem envie novamente.</t>
-        </is>
-      </c>
-      <c r="D273" t="inlineStr"/>
-      <c r="E273" t="inlineStr"/>
-      <c r="F273" t="inlineStr"/>
-      <c r="G273" t="inlineStr"/>
-      <c r="H273" t="inlineStr"/>
-      <c r="I273" t="inlineStr"/>
-      <c r="J273" t="inlineStr"/>
-    </row>
-    <row r="274">
-      <c r="A274" t="inlineStr">
-        <is>
-          <t>select_one confirmo</t>
-        </is>
-      </c>
-      <c r="B274" t="inlineStr">
-        <is>
-          <t>confirmacao_envio</t>
-        </is>
-      </c>
-      <c r="C274" t="inlineStr">
-        <is>
-          <t>Revisei minhas respostas e confirmo o envio.</t>
-        </is>
-      </c>
-      <c r="D274" t="inlineStr"/>
-      <c r="E274" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="F274" t="inlineStr"/>
-      <c r="G274" t="inlineStr"/>
-      <c r="H274" t="inlineStr"/>
-      <c r="I274" t="inlineStr"/>
-      <c r="J274" t="inlineStr"/>
-    </row>
-    <row r="275">
-      <c r="A275" t="inlineStr">
-        <is>
-          <t>end_group</t>
-        </is>
-      </c>
-      <c r="B275" t="inlineStr"/>
-      <c r="C275" t="inlineStr"/>
-      <c r="D275" t="inlineStr"/>
-      <c r="E275" t="inlineStr"/>
-      <c r="F275" t="inlineStr"/>
-      <c r="G275" t="inlineStr"/>
-      <c r="H275" t="inlineStr"/>
-      <c r="I275" t="inlineStr"/>
-      <c r="J275" t="inlineStr"/>
-    </row>
-    <row r="276">
-      <c r="A276" t="inlineStr">
-        <is>
-          <t>end_group</t>
-        </is>
-      </c>
-      <c r="B276" t="inlineStr"/>
-      <c r="C276" t="inlineStr"/>
-      <c r="D276" t="inlineStr"/>
-      <c r="E276" t="inlineStr"/>
-      <c r="F276" t="inlineStr"/>
-      <c r="G276" t="inlineStr"/>
-      <c r="H276" t="inlineStr"/>
-      <c r="I276" t="inlineStr"/>
-      <c r="J276" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -7846,7 +5782,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C278"/>
+  <dimension ref="A1:C271"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12204,372 +10140,253 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>contrib</t>
+          <t>canais</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>recursos</t>
+          <t>whatsapp</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>Recursos</t>
+          <t>WhatsApp</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>contrib</t>
+          <t>canais</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>formacao</t>
+          <t>comunicados_impressos</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>Formação</t>
+          <t>Comunicados impressos</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>contrib</t>
+          <t>canais</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>articulacao_institucional</t>
+          <t>reunioes</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>Articulação institucional</t>
+          <t>Reuniões</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>contrib</t>
+          <t>canais</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>apoio_tecnico</t>
+          <t>redes_sociais</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>Apoio técnico</t>
+          <t>Redes sociais</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>contrib</t>
+          <t>canais</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>mobilizacao_comunitaria</t>
+          <t>alto_falante_radio_local</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>Mobilização comunitária</t>
+          <t>Alto-falante/rádio local</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>contrib</t>
+          <t>canais</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>conhecimentos_tradicionais_locai</t>
+          <t>outro</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>Conhecimentos tradicionais/locais</t>
+          <t>Outro</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>contrib</t>
+          <t>suficiente</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>outro</t>
+          <t>sim</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>Outro</t>
+          <t>Sim</t>
         </is>
       </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>canais</t>
+          <t>suficiente</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>whatsapp</t>
+          <t>parcialmente</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>WhatsApp</t>
+          <t>Parcialmente</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>canais</t>
+          <t>suficiente</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>comunicados_impressos</t>
+          <t>nao</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>Comunicados impressos</t>
+          <t>Não</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>canais</t>
+          <t>suficiente</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>reunioes</t>
+          <t>nao_sabe</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>Reuniões</t>
+          <t>Não sabe</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>canais</t>
+          <t>barr_artic</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>redes_sociais</t>
+          <t>falta_de_contato</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>Redes sociais</t>
+          <t>Falta de contato</t>
         </is>
       </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>canais</t>
+          <t>barr_artic</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>alto_falante_radio_local</t>
+          <t>burocracia</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>Alto-falante/rádio local</t>
+          <t>Burocracia</t>
         </is>
       </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>canais</t>
+          <t>barr_artic</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>outro</t>
+          <t>desconfianca_historico_de_relaca</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>Outro</t>
+          <t>Desconfiança/histórico de relação</t>
         </is>
       </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>suficiente</t>
+          <t>barr_artic</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>sim</t>
+          <t>falta_de_tempo</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Falta de tempo</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>suficiente</t>
+          <t>barr_artic</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>parcialmente</t>
+          <t>outro</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
-        <is>
-          <t>Parcialmente</t>
-        </is>
-      </c>
-    </row>
-    <row r="272">
-      <c r="A272" t="inlineStr">
-        <is>
-          <t>suficiente</t>
-        </is>
-      </c>
-      <c r="B272" t="inlineStr">
-        <is>
-          <t>nao</t>
-        </is>
-      </c>
-      <c r="C272" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-    </row>
-    <row r="273">
-      <c r="A273" t="inlineStr">
-        <is>
-          <t>suficiente</t>
-        </is>
-      </c>
-      <c r="B273" t="inlineStr">
-        <is>
-          <t>nao_sabe</t>
-        </is>
-      </c>
-      <c r="C273" t="inlineStr">
-        <is>
-          <t>Não sabe</t>
-        </is>
-      </c>
-    </row>
-    <row r="274">
-      <c r="A274" t="inlineStr">
-        <is>
-          <t>barr_artic</t>
-        </is>
-      </c>
-      <c r="B274" t="inlineStr">
-        <is>
-          <t>falta_de_contato</t>
-        </is>
-      </c>
-      <c r="C274" t="inlineStr">
-        <is>
-          <t>Falta de contato</t>
-        </is>
-      </c>
-    </row>
-    <row r="275">
-      <c r="A275" t="inlineStr">
-        <is>
-          <t>barr_artic</t>
-        </is>
-      </c>
-      <c r="B275" t="inlineStr">
-        <is>
-          <t>burocracia</t>
-        </is>
-      </c>
-      <c r="C275" t="inlineStr">
-        <is>
-          <t>Burocracia</t>
-        </is>
-      </c>
-    </row>
-    <row r="276">
-      <c r="A276" t="inlineStr">
-        <is>
-          <t>barr_artic</t>
-        </is>
-      </c>
-      <c r="B276" t="inlineStr">
-        <is>
-          <t>desconfianca_historico_de_relaca</t>
-        </is>
-      </c>
-      <c r="C276" t="inlineStr">
-        <is>
-          <t>Desconfiança/histórico de relação</t>
-        </is>
-      </c>
-    </row>
-    <row r="277">
-      <c r="A277" t="inlineStr">
-        <is>
-          <t>barr_artic</t>
-        </is>
-      </c>
-      <c r="B277" t="inlineStr">
-        <is>
-          <t>falta_de_tempo</t>
-        </is>
-      </c>
-      <c r="C277" t="inlineStr">
-        <is>
-          <t>Falta de tempo</t>
-        </is>
-      </c>
-    </row>
-    <row r="278">
-      <c r="A278" t="inlineStr">
-        <is>
-          <t>barr_artic</t>
-        </is>
-      </c>
-      <c r="B278" t="inlineStr">
-        <is>
-          <t>outro</t>
-        </is>
-      </c>
-      <c r="C278" t="inlineStr">
         <is>
           <t>Outra</t>
         </is>

</xml_diff>